<commit_message>
Sinaptogenesi Aginter Press + assi apartheid: 57 nodi, 24 archi, 14 reperti negativi
Nodizza le monografie di ricerca profonda su Aginter Press e sugli assi
dell'apartheid (32 .md in corpus/opera). Hub Aginter/Guerin-Serac; distingue la
liaison certa PIDE-CIA dalla leggenda a fonte unica CIA-Aginter; registra gli
assi nucleare/militare/finanziario dell'apartheid e il contro-campo comunista;
apre la seconda filiera Thiriart -> QUEX/Orion -> Dugin -> Savoini (through-line
al presente). I reperti negativi (Aginter-Asia, mondo arabo, Kissinger, CIA
diretta, Sudafrica) sono registrati come esiti a pieno titolo. Statuto Savona
rispettato; riga 25 del registro delle verifiche.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1548,6 +1548,51 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>SINAPTOGENESI AGINTER PRESS + ASSI DELL'APARTHEID - nodizzazione delle monografie di ricerca profonda (circa trenta schede)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (32 .md) + corpus/diagnostica + repertorio</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>genera 57 nodi, 24 archi, 14 reperti negativi su 6 domini. HUB: Aginter Press (Lisbona 1966; ruolo dottrinale A, operativo B) e Guerin-Serac. SERVIZI: liaison PIDE-CIA (A) distinta dalla leggenda CIA-Aginter (assenza). Le Cercle finanziato da Pretoria (A); unico ponte Aginter-Cercle = contatto Guerin-Serac/Damman 1969 (B). APARTHEID: asse nucleare RFT/URENCO-Rossing, U-Boot HDW/IKL, ISSA Israele-SA (A), obice Bull/G5, broker petroliferi (Chiavelli/Deuss/Rich). SECONDA FILIERA: Thiriart/Jeune Europe -&gt; Mutti/QUEX -&gt; Murelli/Orion -&gt; Dugin -&gt; Savoini/Metropol (through-line al presente).</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Livello A: esistenza e natura di Aginter, Ordre et Tradition, doc 'Notre action politique'; liaison PIDE/DGS-CIA; finanziamento sudafricano a Le Cercle (Khan Committee 1991); ISSA 1975; U-Boot-Affare (Bundestag); ALCORA; contro-campo comunista. Filiere atlantista e antiatlantista tenute distinte.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Livello C e reperti negativi (dichiarati): offerta nucleare Jericho (transazione non avvenuta); Aginter-CIA diretta = leggenda a fonte unica (SDCI-&gt;Laurent-&gt;Christie-&gt;Ganser); Aginter-Sudafrica NON documentato nei 5 paesi; Aginter-Asia/mondo arabo/Kissinger = assenza; FM 30-31B = falso; Delle Chiaie 'membro fondatore' = distorsione (assoluzioni giudiziarie); nesso Aginter-JFK cronologicamente impossibile; 'Shaganovitch' = fabbricazione (vero: Gusev). INCROCI: registro-madre D7 (Aginter, Guerin-Serac, ON, AN, Delle Chiaie, Giannettini gia' registrati); nota su strategia della tensione; nota Minaccia ibrida (Dugin-&gt;Savoini). Vincolo fonti rispettato (no Grokipedia, no 'il manifesto').</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>NODIZZAZIONE CERTIFICATA. Domini: D7, D3, D9, D6, D2, D10.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>ITALIA_NERA_SINAPTOGENESI_AGINTER_APARTHEID.docx + repertorio/ITALIA_NERA_NODI_AGINTER_APARTHEID_INTEGRAZIONE.xlsx</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Approfondimento Aginter: servizi (elenco SDCI), Terza Posizione, assi apartheid del Cono Sud
Seconda tornata di sinaptogenesi (voce 26): 22 nodi, 14 archi, 8 reperti negativi.
Adjudica l'elenco SDCI voce per voce (la voce greca KYP/Plevris e' la meglio
fondata, da fonte primaria; SDECE = matrice non committenza; canale tedesco =
Taubert/Kampfbund non BND; DGS = Paladin post-1974). Registra la distinzione tra
Aginter e Terza Posizione (nessun nesso organico), la verita' giudiziaria di
Piazza Fontana (assoluzioni definitive, Cassazione 2005), e gli assi apartheid
del Cono Sud (Paraguay-Vorster, Cile skunk status/Cardoen, Argentina CAL/P2,
Brasile Decreto 1985/MNU). Statuto Savona rispettato; niente Grokipedia ne'
il manifesto come fonti.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1593,6 +1593,51 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>SINAPTOGENESI AGINTER (APPROFONDIMENTO) - servizi dell'elenco SDCI, Terza Posizione, assi apartheid del Cono Sud</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (33 .md) + corpus/diagnostica + repertorio</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>aggiunge 22 nodi, 14 archi, 8 reperti negativi alla voce 25. SERVIZI (elenco SDCI voce per voce): la voce GRECA (KYP/Plevris) e' la meglio fondata, da fonte primaria (lettera Guerin-Serac 3 dic 1973, atti Brescia); SDECE = matrice/provenienza non committenza; canale tedesco = Taubert/Kampfbund, non BND; Strauss != BND; DGS spagnola = Paladin/Skorzeny (post-1974). USA: liaison CIA-PIDE certa, 'CIA creo' Aginter' = eccesso di Ganser; rete Digilio/US Navy = ipotesi istruttoria. TERZA POSIZIONE (Fiore/Adinolfi/Dimitri 1978): nessun nesso organico con Aginter. ASSI: Paraguay-Vorster 1975, Rheinmetall-Durban; Cile skunk status/Cardoen; Argentina CAL 1980/P2 (Massera, Suarez Mason); Brasile Decreto 1985/MNU/Abdias.</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Livello A: visite di Stato Stroessner-Vorster; P2 in Argentina (Massera, Suarez Mason); matrice SDECE/OAS del personale. Livello B: lettera KYP 1973; viaggio Grecia 1968; Taubert/Kampfbund; Rheinmetall-Paraguay-Durban; CAL 1980; Cardoen 'Made in Chile'; golpe Garcia Meza (Delle Chiaie+Barbie); mandanti Bologna (sentenza Bellini 2022, Cavallini def. 2025).</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Reperti negativi dichiarati: Piazza Fontana = assoluzioni definitive (Cassazione 2005 n.21998; Digilio 'inattendibile'); Aginter-Terza Posizione = nessun nesso organico (cronologia; TP assente dagli atti Salvini); 'CIA creo' Aginter' = eccesso tesistico; von Leers cofondatore Paladin = impossibile (morto 1965); Strauss=BND non dimostrato; presenza SA a WACL Asuncion 1979 / Archivio del Terrore = assente; Cile in 'Pia Vesta' = assente (solo Peru' e Panama); Condor-Sudafrica = sistemi paralleli. INCROCI: voce 25 (prima tornata); note su strategia della tensione; registro-madre D4 (P2) e D7.</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>NODIZZAZIONE CERTIFICATA. Domini: D7, D3, D2, D9, D6, D4.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>ITALIA_NERA_SINAPTOGENESI_AGINTER_APARTHEID_2.docx + repertorio/ITALIA_NERA_NODI_AGINTER_APARTHEID_APPROFONDIMENTO.xlsx</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Triangolazione dei nodi attorno a Vladimir Putin
Voce 27: fa convergere sul nodo-hub Putin 24 nodi, 15 archi, 8 reperti negativi.
Fascio finanza/energia (Ozero/Bank Rossiya, Yukos/lodo Aja, MENATEP, Gazprom,
tagli gas): archi solidi. Fascio guerra cognitiva (IRA/Prigozhin -> Doppelganger
-> Tenet) con proiezione in Italia (Lombardia-Russia/Savoini, Metropol): solido.
Filiera eurasiatista (Thiriart -> Murelli/Orion -> Dugin -> Malofeev): genealogia
d'idee, non catena di comando. Reperto negativo maggiore: la galassia
Aginter/apartheid NON converge su Putin (atlantista, sciolta 1974); unico ponte
legittimo = eco di metodo (strategia della tensione = falsa bandiera). Statuto
Savona rispettato su persone viventi/indagate (Metropol non e' reato; influenza
Dugin contestata; 'portafoglio' allegazione). Niente Grokipedia ne' il manifesto.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1638,6 +1638,51 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE DEI NODI ATTORNO A VLADIMIR PUTIN - convergenza dell'arco russo, della filiera eurasiatista e (in negativo) della galassia Aginter</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica + repertorio (nodi dell'intera sessione)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>fa convergere sul nodo-hub Putin 24 nodi, 15 archi, 8 reperti negativi. FASCIO 1 (solido): catena finanza/energia - Ozero/Kovalchuk/Bank Rossiya; espropriazione Yukos e lodo Aja (~50 mld); pivot MENATEP/Khodorkovsky; Gazprom renazionalizzata; tagli gas 2006/2009; RosUkrEnergo/Firtash/Mogilevich. FASCIO 2 (solido): guerra cognitiva - IRA/Prigozhin -&gt; Doppelganger -&gt; Tenet/Pravda; proiezione in Italia via Lombardia-Russia/Savoini e affare Metropol (Dugin in trattativa). FASCIO 3 (genealogia, non comando): filiera eurasiatista Thiriart -&gt; Murelli/Orion -&gt; Dugin -&gt; Malofeev/Komov.</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Livello A: espropriazione Yukos/lodo Aja; sanzioni a Bank Rossiya (2014); renazionalizzazione Gazprom; tagli del gas; IRA/Doppelganger; invasione Ucraina (2022); esistenza dell'audio Metropol e di Lombardia-Russia; repressione (Navalny, Dossier Center).</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Livello B/C e reperti negativi: la galassia AGINTER/APARTHEID NON converge su Putin (assenza di riscontro: Aginter atlantista, sciolta 1974, antipodo della filiera filorussa); Thiriart-&gt;Dugin-&gt;Putin = genealogia di idee, non catena di comando; Dugin 'cervello di Putin' = semplificazione; Metropol = negoziazione documentata != reato (archiviazione 2023; Savoini indagato non condannato; Salvini non imputato); 'portafoglio di Putin'/Roldugin = allegazione; Khodorkovsky = persecuzione accertata ma origine fortuna contestata; unico ponte legittimo Aginter-Putin = ECO DI METODO (strategia della tensione = falsa bandiera), non linea di comando. INCROCI: voci 5-24 della sessione (arco russo) + voci 25-26 (Aginter/apartheid). Vincolo fonti rispettato.</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE CERTIFICATA. Domini: D2, D3, D6, D7, D8, D9, D10.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>ITALIA_NERA_TRIANGOLAZIONE_PUTIN.docx + repertorio/ITALIA_NERA_TRIANGOLAZIONE_PUTIN.xlsx</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Verifica biografica di Vladimir Putin dalla gioventu' (fonti online)
Voce 28: certifica la spina biografica del nodo-hub Putin in 17 tappe datate,
riscontrate su fonti online indipendenti e incrociate (Wikipedia, Britannica,
kremlin.ru bilanciata, Wilson Center, RFE/RL, TBIJ, Havighurst Center, IAI).
Dalla nascita a Leningrado (1952) e dall'infanzia di cortile (sambo/judo) alla
Facolta' di Giurisprudenza e a Sobchak, al KGB (1975) e a Dresda (1985-90), fino
allo staff di Sobchak, all'FSB (1998) e alla presidenza (2000). Statuto
rispettato: tessera Stasi precisata come agevolazione d'accesso (non
appartenenza); commissione Salye 1992 = difetto di controllo, non corruzione
personale (allegazione != sentenza). Radice biografica del nodo triangolato
(voce 27). Niente Grokipedia ne' il manifesto.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1683,6 +1683,51 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>VERIFICA BIOGRAFICA DI VLADIMIR PUTIN DALLA GIOVENTU' - documentazione e certificazione su fonti online</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica + repertorio (verifica online)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>certifica la spina biografica del nodo-hub Putin in 17 tappe datate, riscontrate su fonti indipendenti reperite in rete e incrociate. Nascita a Leningrado (7 ott 1952; kommunalka vicolo Baskov; padre reduce ferito, due fratelli morti); infanzia di cortile, sambo/judo (First Person); Giurisprudenza a Leningrado (1970-75, docente Sobchak); KGB dal 1975 (scuola di Okhta); Dresda 1985-90; ritiro col grado di tenente colonnello; staff di Sobchak; Comitato Relazioni Esterne 1991; primo vicesindaco 1994; Mosca 1996; direttore FSB 1998; premier ago 1999; presidente ad interim 31 dic 1999; eletto 26 mar 2000.</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Livello A: tutti i fatti biografici e di carriera (nascita, scuola, laurea, KGB, Dresda, staff Sobchak, ascesa a Mosca, FSB, premier, presidenza), riscontrati su Wikipedia, Britannica, kremlin.ru (bilanciata), GlobalSecurity, Russia Beyond, Wilson Center, RFE/RL, TBIJ, Havighurst Center (Miami), IAI.</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Livello B e precisazioni (fragilita'): l'autonarrazione della gioventu' rissosa ('First Person') e' segnalata come tale; la TESSERA STASI di Dresda e' agevolazione d'accesso documentata, NON appartenenza alla Stasi (precisazione Wilson Center contro la 'sensazione stampa'); la COMMISSIONE SALYE (1992) contesto' a Putin un DIFETTO DI CONTROLLO, non una corruzione personale, e non produsse alcun procedimento (allegazione != sentenza). INCROCIO: radice biografica del nodo-hub gia' triangolato (voce 27). Verifica online, non collazione; fonte ufficiale usata ma bilanciata. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>VERIFICA CERTIFICATA. Domini: D2, D3.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>ITALIA_NERA_VERIFICA_BIOGRAFICA_PUTIN.docx + repertorio/ITALIA_NERA_VERIFICA_BIOGRAFICA_PUTIN.xlsx</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Triangolazione integrale: Vladimir Putin contro tutto il corpus
Voce 31: rieffettua la triangolazione del nodo-hub sull'intero corpus, per
dominio. 28 nodi sui dieci Domini di Potere + radice biografica (voci 28-30),
13 archi maestri, 10 reperti negativi. Cuore duro D6: EUB->BoNY->MENATEP/Yukos,
Bank Rossiya, Gazprom/gas. D8+D2: guerra cognitiva e proiezione in Italia. D1:
Tambov e Mogilevich al grado dell'indagine. D7/D10: filiera eurasiatista come
genealogia. Reperti negativi maestri: Aginter/apartheid, Terza Posizione e P2
NON convergono; Thiriart->Dugin = genealogia non comando; Metropol non e' reato;
Salye difetto di controllo; Tambov/SPAG/Ozero = indagine. Statuto rispettato in
ogni dominio; niente Grokipedia ne' il manifesto.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1818,6 +1818,51 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE INTEGRALE - Vladimir Putin contro tutto il corpus, per dominio</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica + repertorio (intero corpus della sessione)</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>rieffettua la triangolazione del nodo-hub sull'intero corpus, disponendo 28 nodi per i dieci Domini di Potere + la radice biografica, con 13 archi maestri e 10 reperti negativi. RADICE: spina 1952-2000 (voci 28-30). CUORE DURO (D6): EUB-&gt;BoNY-&gt;MENATEP/Yukos/lodo Aja; Ozero/Bank Rossiya; Gazprom/RosUkrEnergo/tagli gas. D8+D2: IRA/Doppelganger/Tenet + Lombardia-Russia/Metropol/accordo Lega + invasione Ucraina. D1: Tambov/Kumarin e Mogilevich (cerniera). D7/D10: filiera eurasiatista Thiriart-&gt;Murelli-&gt;Dugin-&gt;Malofeev (genealogia). D9: repressione (Navalny, Dossier Center).</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Livello A: radice biografica; catena finanza EUB-BoNY-MENATEP/Yukos; Bank Rossiya (sanzioni 2014); Gazprom/tagli gas; IRA/Doppelganger; Metropol (esistenza) e accordo Lega-Russia Unita; invasione Ucraina; persecuzione oppositori. Cornice D3: KGB/FSB, siloviki, Ozero.</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Reperti negativi maestri: GALASSIA AGINTER/APARTHEID non converge (antipodo atlantista; solo eco di metodo); TERZA POSIZIONE distinta; LOGGIA P2 non converge (rete italo-argentina di altra epoca; analogia di forma, non nesso); Thiriart-&gt;Dugin = genealogia non comando; Metropol negoziazione non reato; Salye difetto di controllo non corruzione; Bank Rossiya via casino'/SPAG/Tambov/Ozero = indagine; 'portafoglio'/Roldugin = allegazione; Khodorkovsky persecuzione accertata ma fortuna contestata. INCROCI: voci 25-30 (Aginter, arco russo, biografia). Vincolo fonti rispettato.</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE INTEGRALE CERTIFICATA. Domini: D1, D2, D3, D4, D6, D7, D8, D9, D10 + radice biografica.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>ITALIA_NERA_TRIANGOLAZIONE_INTEGRALE_PUTIN.docx + repertorio/ITALIA_NERA_TRIANGOLAZIONE_INTEGRALE_PUTIN.xlsx</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Prima triangolazione: Putin e la galassia nera del corpus
Voce 32: triangola Putin con Aginter, Sudafrica, Brighton Beach, Sud America,
estrema destra, nazi-fascismo. Un solo ponte reale e documentato - non
ideologico ma criminale-finanziario-energetico: Brighton Beach -> Ivankov ->
Mogilevich -> riciclaggio Bank of New York -> RosUkrEnergo/Firtash -> Gazprom
(convergenza sistemica, non comando personale). Secondo ponte: estrema destra
come genealogia (Thiriart -> Dugin). Terzo filo: eco di metodo (strategia della
tensione -> guerra cognitiva). Grande campo negativo dichiarato: Aginter,
apartheid Sudafrica, Sud America neofascista e diaspora nazista storica NON
convergono (antipodo atlantista di Guerra Fredda). Statuto rispettato; niente
Grokipedia ne' il manifesto.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1863,6 +1863,51 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>PRIMA TRIANGOLAZIONE Putin e la GALASSIA NERA (Aginter, Sudafrica, Brighton Beach, Sud America, estrema destra, nazi-fascismo)</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica + repertorio (schede e documentazioni caricate e generate)</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>triangola Putin con i temi neri del corpus. UN SOLO PONTE REALE E DOCUMENTATO, non ideologico ma criminale-finanziario-energetico: Brighton Beach -&gt; Ivankov (Solntsevskaya) -&gt; Mogilevich (FBI most wanted; pago' un giudice per Ivankov nel 1991) -&gt; riciclaggio Bank of New York (YBM Magnex/Benex, 1998-99, miliardi) -&gt; RosUkrEnergo/Firtash (cablogramma 2010: 'partito con l'aiuto di Mogilevich') -&gt; Gazprom. Secondo ponte: estrema destra come GENEALOGIA (Thiriart-&gt;Murelli/Orion-&gt;Dugin-&gt;Malofeev/Komov/Lombardia-Russia). Terzo filo: ECO DI METODO (strategia della tensione di Aginter -&gt; guerra cognitiva).</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Livello A: schema di riciclaggio Bank of New York (miliardi; condanne 2000). Livello B: Brighton Beach/Ivankov/Mogilevich (atti giudiziari/FBI); RosUkrEnergo/Firtash-Mogilevich (cablogramma 2010); convergenza sistemica crimine-finanza-gas con lo Stato-cerchia; genealogia eurasiatista; eco di metodo; strumentalizzazione odierna del nazi-fascismo (Movimento Imperiale Russo, terrorista USA 2020).</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>GRANDE CAMPO NEGATIVO (assenza di riscontro): Aginter Press (atlantista, sciolta 1974); Sudafrica apartheid (assi occidentali; il solo filo sovietico e' il CONTROCAMPO che armava l'ANC, epoca pre-Putin, lato opposto); Sud America neofascista (Condor, Delle Chiaie, Garcia Meza, CAL, Stroessner = Guerra Fredda); diaspora nazista storica (Skorzeny, Paladin, von Leers, ratlines = Guerra Fredda occidentale). CAUTELA: il ponte di Brighton Beach e' CONVERGENZA SISTEMICA, NON comando personale provato di Putin su Mogilevich; Thiriart-&gt;Dugin = genealogia non comando; nazi-fascismo odierno = inversione, non continuita'. INCROCI: voci 25-31. Vincolo fonti rispettato.</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE FOCALIZZATA CERTIFICATA. Domini: D1, D6, D7, D8, D10.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>ITALIA_NERA_TRIANGOLAZIONE_PUTIN_GALASSIA_NERA.docx + repertorio/ITALIA_NERA_TRIANGOLAZIONE_PUTIN_GALASSIA_NERA.xlsx</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Triangolazione: le Cinque Famiglie (Censimento), Brighton Beach e Putin
Voce 33: triangola le Cinque Famiglie di Cosa Nostra USA (dal Censimento della
criminalita' organizzata) con l'arco eurasiatico verso Putin. Nesso documentato:
lo schema della benzina degli anni Ottanta - Agron/Balagula e le 'burn
companies'; le Cinque Famiglie imposero il 'Family tax' di 2 centesimi/gallone
(Colombo/Franzese, Lucchese/Furnari, Genovese/Galizia). Cerniera russa: da
Balagula a Ivankov/Mogilevich -> Bank of New York -> RosUkrEnergo/gas -> Gazprom.
Reperto negativo centrale: le Cinque Famiglie NON convergono direttamente su
Putin, separate da due cerniere; la catena russa non risale a un suo comando
personale (convergenza di milieu). Asse laterale distinto: Gambino-'ndrangheta
(New Bridge). Statuto rispettato; niente Grokipedia ne' il manifesto.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1908,6 +1908,51 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE 5 FAMIGLIE (Censimento Criminalita') - mafia russa di Brighton Beach - Putin</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica + repertorio (nodi D1 dal Censimento + arco eurasiatico)</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>triangola le Cinque Famiglie di Cosa Nostra USA (Genovese, Gambino, Lucchese, Bonanno, Colombo; dal Censimento globale della criminalita') con l'arco che arriva a Putin. NESSO DOCUMENTATO: lo schema della benzina degli anni Ottanta - Agron (Leningrado) e Balagula (associato di Lucchese e Colombo) con le 'burn companies' (~150 mln di carburante/mese); le Cinque Famiglie imposero il 'Family tax' di 2 centesimi/gallone (maggiore introito dopo la droga); Colombo (Franzese/Sciortino), Lucchese (mediazione Furnari), Genovese (ramo Galizia). CERNIERA RUSSA: da Balagula la regia passa a Ivankov (Solntsevskaya) e Mogilevich -&gt; riciclaggio Bank of New York -&gt; RosUkrEnergo/Firtash -&gt; Gazprom -&gt; orbita statale.</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Livello A: schema della benzina e 'Family tax' (RICO, testimonianze Franzese); Balagula associato di Lucchese/Colombo; riciclaggio Bank of New York. Livello B: subentro Ivankov/Mogilevich; RosUkrEnergo/Firtash-Mogilevich (cablogramma 2010); convergenza sistemica gas-Stato.</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>REPERTO NEGATIVO CENTRALE: le Cinque Famiglie NON convergono direttamente su Putin - ne sono separate da DUE CERNIERE (1. mafia russa di Brighton Beach; 2. complesso crimine-finanza-gas su Mogilevich); e neppure la catena russa risale a un comando personale di Putin (convergenza di milieu, non ordine). Cosa Nostra italiana e mafia russa = 'alleanza scomoda' (tributo/coordinamento, non fusione); il 'Family tax' e' crimine di strada anni Ottanta, precedente all'era Putin. ASSE LATERALE distinto: Gambino-'ndrangheta (Ursino, New Bridge), italo-italiano, estraneo alla catena russa. Mafie del Censimento tenute distinte. INCROCI: nodi D1 (Censimento); note 9 e 14; voce 32. Vincolo fonti rispettato.</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE CERTIFICATA. Domini: D1, D6, D2.</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>ITALIA_NERA_TRIANGOLAZIONE_5FAMIGLIE_PUTIN.docx + repertorio/ITALIA_NERA_TRIANGOLAZIONE_5FAMIGLIE_PUTIN.xlsx</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Armi e bossoli del caso Moro: 20 blocchi di ricerca, Excel di servizio
Voce 35: ricognizione balistica di via Fani (16.3.1978) e dell'omicidio Moro
(9.5.1978). Via Fani: 91 bossoli 9 Para repertati (93 colpi per la Scientifica,
2 di Iozzino; 87 in esami successivi - discrepanza dichiarata); ripartizione
perizia 1978: 49+22+5+3+8+4 su due FNAB-43, TZ-45, Beretta M12, S&W e Beretta 51;
munizioni GFL 9M38 con 30 bossoli senza data; il 'super-killer' smontato da
Salza-Benedetti; ipotesi dell'arma non identificata (Comm. Moro 2). 9 maggio:
Walther PPK 9 corto (inceppata) + Skorpion vz.61 7,65 (raffica di 11, varianti
9/12); catena della Skorpion di via Dogali (Tarantelli, Conti, Ruffilli; nesso
Acca Larentia; provenienza Sanremo 1971/Jimmy Fontana, passaggio alle BR mai
chiarito). Excel a 6 fogli con gradi e apparato fonti; discrepanze dichiarate.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1998,6 +1998,51 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>ARMI E BOSSOLI DEL CASO MORO (via Fani 16.3.1978 + omicidio 9.5.1978) - 20 blocchi di ricerca mirati, Excel di servizio</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>repertorio (foglio di servizio balistico)</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>VIA FANI: 91 bossoli cal. 9 Parabellum repertati (93 colpi sparati per la Scientifica, di cui 2 di Iozzino; 87 bossoli in esami successivi - discrepanza dichiarata). Ripartizione perizia 1978 (Ugolini-Jadevito-Lopez): 49 (FNAB-43 o Sten) + 22 (seconda FNAB-43) + 5 (TZ-45) + 3 (Beretta M12) + 8 (pistola S&amp;W cal.9) + 4 (Beretta mod.51) = 91. Fucilieri (memoriali): Morucci e Bonisoli (FNAB-43), Fiore (M12, inceppata), Gallinari (TZ-45); piu' inceppamenti; unica reazione: Iozzino, 2 colpi. Munizioni G.F.L. 9M38 (Fiocchi); 30 bossoli su 87 SENZA anno di fabbricazione. 9 MAGGIO: Walther PPK 9 corto con silenziatore (inceppata) + Skorpion vz.61 7,65 (raffica di 11 colpi, varianti 9/12); esecutore Moretti; Renault 4 rossa targa Roma N57686.</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Livello A: ripartizione della perizia 1978; 91 bossoli; esiti Salza-Benedetti (il 'super-killer' dei 49 colpi NON confermato; solo 6 a segno); marchio GFL 9M38 e cartucce senza data; armi del 9 maggio; sequestro della Skorpion in via Dogali (15.6.1988) e catena balistica Tarantelli-Conti-Ruffilli.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Fragilita' e ipotesi dichiarate: discrepanza 87/91/93; arma NON identificata (Comm. Moro 2: nessun proiettile 9 Para dalle armi sequestrate); interpretazione delle cartucce senza data (forniture non convenzionali/export) = ipotesi peritale, replicata da Fiocchi; identita' Skorpion via Dogali = arma di Moro (B) e nesso Acca Larentia (B); provenienza Skorpion: Jimmy Fontana, Sanremo feb. 1971, ceduta 1977, passaggio alle BR MAI chiarito (C); numero esatto bossoli 7,65/9 corto di via Caetani: da atti (C); provenienza armi lunghe BR non accertata. INCROCI: registro-madre D7; note sulla strategia della tensione. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>RICOGNIZIONE BALISTICA CERTIFICATA (con discrepanze dichiarate). Domini: D7, D3.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>repertorio/ITALIA_NERA_MORO_ARMI_E_BOSSOLI.xlsx (Excel di servizio, 6 fogli)</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Moro esecuzione (9 mag 1978): armi e bossoli sul corpo, perimetro ristretto (voce 36)
Excel di servizio a 6 fogli sulle sole armi/colpi dell'esecuzione nel
covo (Walther PPK 9 corto inceppata + Skorpion vz.61 7,65, silenziatore),
undici fori al torace, otto proiettili ritenuti, discrepanze e statuto
Savona; esclude i novantuno bossoli di via Fani (voce 35). Registro
verifiche aggiornato a voce 36.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2043,6 +2043,51 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>ARMI E BOSSOLI USATI DIRETTAMENTE SU ALDO MORO NELL'ESECUZIONE (9 maggio 1978) - perimetro ristretto: SOLO il covo/garage, ESCLUSO il rapimento di via Fani</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>repertorio (foglio di servizio balistico - esecuzione)</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>DUE ARMI sul corpo: (uno) Walther PPK cal. 9 corto (9x17 / .380 ACP), con silenziatore, esploso il primo colpo e subito INCEPPATA (uno-due colpi), MAI ritrovata; (due) mitra cecoslovacco Skorpion vz.61 cal. 7,65 Browning (.32 ACP), con silenziatore, raffica di undici colpi (varianti in perizia dieci/dodici). Esecutore materiale indicato: Mario Moretti. ESITO SUL CORPO: undici fori d'ingresso al torace (perizia necroscopica; perizie successive parlano di piu' colpi); otto proiettili ritenuti nel corpo, solo tre fuoriusciti. Corpo nel bagagliaio di una Renault 4 rossa targata Roma N57686, via Michelangelo Caetani. Il garage/box: via Camillo Montalcini. RIS Parma 2017: Moro colpito di fronte e in posizione eretta o semi-eretta, non rannicchiato nel bagagliaio come da versione BR.</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Livello A: le due armi (Walther PPK 9 corto inceppata + Skorpion 7,65); il silenziatore; la Renault 4 e la targa; via Caetani e via Montalcini; il sequestro della Skorpion in via Dogali (15.6.1988) con la catena balistica che la lega ai colpi su Moro; la rilettura RIS 2017. Livello B: numero dei colpi Skorpion (undici, con varianti dieci/dodici a seconda della perizia); attribuzione a Moretti come esecutore.</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Fragilita' e ipotesi dichiarate: NUMERO ESATTO DEI BOSSOLI per calibro (7,65 Browning e 9 corto) raccolti nel covo/garage = DA VERIFICARE sugli atti processuali (C) - la Walther si inceppa dopo il primo colpo, quindi i bossoli 9 corto sono pochissimi; discrepanza undici/dodici colpi tra perizia necroscopica e perizie successive; la Walther PPK non fu MAI ritrovata (arma non periziabile fisicamente); provenienza e passaggio della Skorpion alle BR non pienamente chiariti (C). PERIMETRO DICHIARATO: questa voce isola i colpi/bossoli dell'ESECUZIONE (garage, sul corpo) ed ESCLUDE i novantuno bossoli cal. 9 Parabellum di via Fani (rapimento, gia' alla voce trentacinque). INCROCI: voce trentacinque (quadro completo Moro); registro-madre D7. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>RICOGNIZIONE BALISTICA DELL'ESECUZIONE CERTIFICATA (perimetro ristretto, con discrepanze dichiarate). Domini: D7, D3.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>repertorio/ITALIA_NERA_MORO_ESECUZIONE_ARMI_E_BOSSOLI.xlsx (Excel di servizio, 6 fogli)</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ricognizione Walther PPK 9 corto pre-1978 in Italia: esito negativo dichiarato (voce 37)
Dieci blocchi di ricerca sugli omicidi italiani fino al 1977: nessuno
attribuito a una Walther PPK 9 corto nelle fonti aperte. Censiti otto
casi con arma accertata; unica adiacenza tipologica il caso Walter
Rossi (Beretta M34 9 corto con attacco silenziatore, mai ritrovata),
registrata come convergenza di tipologia e non come ponte. Registro
verifiche aggiornato a voce 37 (grigio, reperto negativo).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -31,7 +31,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,11 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -66,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -78,6 +83,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -445,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2088,6 +2096,51 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>RICOGNIZIONE: omicidi in Italia FINO AL 1977 con Walther PPK calibro 9 corto (escluso il caso Moro) - dieci blocchi di ricerca, esito negativo dichiarato</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>repertorio (foglio di servizio balistico - ricognizione)</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>ESITO CENTRALE (REPERTO NEGATIVO): nessun omicidio in Italia fino al 1977 risulta attribuito, nelle fonti aperte consultate, a una Walther PPK cal. 9 corto. Casi esaminati con arma accertata: Calabresi 1972 (S&amp;W .38), Mantakas 1975 (.38 fatale / 7,65 rinvenuta), Alcamo Marina 1976 (cal. 9 'militare' matricola abrasa), Occorsio 1976 (mitraglietta 9 Para), Casalegno 1977 (Nagant 7,62, lo stesso di Croce), Walter Rossi 1977 (Beretta M34 cal. 9 CORTO matricola abrasa CON ATTACCO SILENZIATORE, mai ritrovata). Pedenovi 1976 e Ciotta 1977: calibro non specificato nelle fonti aperte. Contesto: in Italia il 9 corto e' il calibro della Beretta M34 d'ordinanza (PS/CC/GdF), non della PPK.</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Livello A: armi accertate dei singoli casi (Calabresi, Casalegno/Croce, Occorsio, Alcamo Marina); il quadro del 9 corto italiano (M34 d'ordinanza, soglia civile). Livello B: Beretta M34 9 corto con attacco silenziatore per Walter Rossi (inchiesta e atti di parte, procedimento archiviato).</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Fragilita' dichiarate: reperto negativo, NON prova d'inesistenza (perizie d'epoca non integralmente digitalizzate; calibri di Pedenovi e Ciotta non reperiti in rete = giallo); la PPK di Moro MAI ritrovata, quindi nessuna comparazione balistica con delitti precedenti fu mai possibile (limite strutturale della prova, arancio). NON-INFERENZA dichiarata: il parallelo tipologico col caso Walter Rossi (9 corto + silenziatore + arma sparita, Roma, otto mesi prima di via Montalcini) registra una convergenza di tipologia, NON un'identita' d'arma ne' un ponte tra i due fatti. Direzione d'archivio: perizie balistiche originali e casellario balistico storico PS/CC (C). INCROCI: voci 35-36 (balistica Moro). Vincolo fonti rispettato (no Grokipedia, no il manifesto). Ricerca a finalita' difensiva/storiografica.</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>RICOGNIZIONE CON ESITO NEGATIVO DICHIARATO (assenza di riscontro registrata come risultato). Domini: D7, D3.</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>repertorio/ITALIA_NERA_WALTHER_PPK_PRE1978_RICOGNIZIONE.xlsx (Excel di servizio, 5 fogli)</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ricognizione Beretta M34 9 corto pre-1978 in Italia: esito parziale (voce 38)
Gemella della voce 37 (Walther PPK): undici blocchi di ricerca sugli
omicidi italiani fino al 1977. Un positivo probabile (Walter Rossi,
Roma 30.9.1977: M34 matricola abrasa con attacco silenziatore, mai
ritrovata), tre candidati d'ordinanza non modellizzati (Mantini,
Alcamo Marina, Lorusso), tredici casi censiti in tutto. Registro
verifiche aggiornato a voce 38 (giallo, esito parziale).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2141,6 +2141,51 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>RICOGNIZIONE: omicidi in Italia FINO AL 1977 con Beretta M34 calibro 9 corto (escluso il caso Moro) - undici blocchi di ricerca, esito parziale - gemella della voce 37 (Walther PPK)</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>repertorio (foglio di servizio balistico - ricognizione)</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>ESITO PARZIALE: UN caso positivo probabile - omicidio di WALTER ROSSI (Roma, 30.9.1977): Beretta M34 cal. 9 corto, matricola abrasa, ATTACCO PER SILENZIATORE, mai ritrovata (Alibrandi/Fioravanti, FdG/futuri NAR; procedimento archiviato). TRE candidati 'd'ordinanza' con modello non accertato: Lorusso 1977 (Beretta cal. 9 del carabiniere Tramontani, proiettile mai comparabile), Alcamo Marina 1976 (cal. 9 'militare' matricola abrasa, caso Gulotta), Mantini 1975 (colpo ravvicinato d'ordinanza, Tuzzolino). NEGATIVI con arma accertata diversa: Calabresi (S&amp;W .38), Spampinato (S&amp;W), Campanile (due 7,65), Occorsio (9 Para), Masi (.22 blindato), Casalegno/Croce (Nagant 7,62), Reggio Emilia 1960 (mitra e moschetti). Non modellizzati in rete: Cavallero 1967, Di Rosa 1976, Dalmine 1977.</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Livello A: quadro d'ordinanza della M34 (Regio Esercito/EI/CC; PS fino ai primi anni Sessanta; GdF fino agli anni Novanta); armi accertate dei casi negativi. Livello B: M34 di Walter Rossi (fonte d'inchiesta e atti di parte - l'arma non fu mai sequestrata ne' periziata, quindi il grado NON sale ad A). Nota extra-perimetro: Gandhi 1948 (l'omicidio piu' celebre con M34, fuori Italia).</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Fragilita' dichiarate: fascia 'd'ordinanza' (Mantini/Alcamo/Lorusso) con modello non negli atti pubblici e comparazione balistica mancata in tutti e tre i casi - stessa fragilita' strutturale della PPK di Moro (voce 37); calibri non modellizzati in rete per Cavallero, Pedenovi, Ciotta, Di Rosa, Dalmine (chiudibili solo in archivio, C). PONTE dichiarato con la voce 37: Walter Rossi e' insieme il positivo della M34 e l'unica adiacenza tipologica della PPK di via Montalcini (9 corto + silenziatore + arma sparita, stessa citta', otto mesi prima) - convergenza di tipologia, NON identita' d'arma. INCROCI: voci 35-37. Vincolo fonti rispettato (no Grokipedia, no il manifesto). Ricerca a finalita' difensiva/storiografica.</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>RICOGNIZIONE CON ESITO PARZIALE (un positivo probabile, tre candidati, resto negativo). Domini: D7, D3.</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>repertorio/ITALIA_NERA_BERETTA_M34_PRE1978_RICOGNIZIONE.xlsx (Excel di servizio, 5 fogli)</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ricognizione Walther PPK 9 corto dal 1978 in poi: unico caso Moro (voce 39)
Chiude il trittico balistico (voci 37-38-39): nove blocchi di ricerca
sugli omicidi italiani dal 1978. Unico positivo l'esecuzione Moro
(caso ancora); candidato d'identita' la PPK/S ricalibrata di via
Silvani (reperto 47/18, mai verificata); negativi accertati da Acca
Larentia a Gucci. La PPK risulta un unicum balistico nella storia
italiana. Registro verifiche aggiornato a voce 39 (grigio).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2186,6 +2186,51 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>RICOGNIZIONE: omicidi in Italia DAL 1978 IN POI con Walther PPK calibro 9 corto - nove blocchi di ricerca - terza ricognizione della serie balistica (chiude il trittico con le voci 37-38)</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>repertorio (foglio di servizio balistico - ricognizione)</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>ESITO: l'UNICO omicidio italiano dal 1978 in poi attribuito a una Walther PPK cal. 9 corto resta l'esecuzione di ALDO MORO (9.5.1978, caso ancora, gia' voci 35-36). Oltre Moro: NESSUN altro caso nelle fonti aperte. CANDIDATO D'IDENTITA' (C): nel covo BR di via Silvani fu sequestrata una PPK/S nata 7,65 e RICALIBRATA 9 corto, matricola abrasa riemersa con acidi che danneggiarono la rigatura (reperto 47/18) - candidata come arma di via Montalcini secondo la ricostruzione Cucchiarelli, MAI verificata balisticamente ('mai riconosciuta' anziche' 'mai ritrovata'). NEGATIVI accertati: Acca Larentia (7,65/Skorpion), Fausto e Iaio (Beretta 34 ricalibrata 7,65 CON SILENZIATORE, proiettili spariti, indagini riaperte), Pecorelli (7,65 Gevelot), Mattarella (.38 Special/Colt Cobra), Amato (revolver), Gucci 1995 (7,65 con silenziatore artigianale). Tobagi: calibro non modellizzato (giallo).</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Livello A: armi accertate dei casi negativi; il caso ancora Moro. Livello B: quadro Fausto e Iaio (perizia citata da fonti aperte; proiettili spariti). CONCLUSIONE DEL TRITTICO (voci 37-38-39): il 9 corto italiano e' territorio della Beretta M34; la Walther PPK non ha scia ne' prima ne' dopo Moro - l'arma dell'esecuzione e' un UNICUM balistico nella storia italiana, il che rende provenienza e sparizione ancora piu' significative.</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Fragilita' dichiarate: candidato via Silvani = ricostruzione di parte su atti, mai verificata (C); calibro Tobagi non reperito in rete (giallo); indagini Fausto e Iaio riaperte (2025) con ricerca di collegamenti balistici col caso Pecorelli - quadro in evoluzione. Non-inferenza: le adiacenze del silenziatore (Fausto e Iaio, Gucci) restano convergenze di tipologia, nessun ponte balistico accertato con la PPK di Moro. INCROCI: voci 35-38. Vincolo fonti rispettato (no Grokipedia, no il manifesto). Ricerca a finalita' difensiva/storiografica.</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>RICOGNIZIONE CON ESITO NEGATIVO OLTRE L'ANCORA (unico caso: Moro). Domini: D7, D3.</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>repertorio/ITALIA_NERA_WALTHER_PPK_POST1978_RICOGNIZIONE.xlsx (Excel di servizio, 5 fogli)</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Arsenale Sardo BR (Lula 1982): ricognizione armi e triangolazione col corpus (voce 40)
Ritrovamento di Lula (Monte Albo-Monte Pitzinnu, febbraio 1982) su
indicazione di Savasta, custodia Barbagia Rossa: inventario certificato
con discrepanze del paragrafo circolante dichiarate. Filiera OLP
documentata (viaggio del Papago 1979, consegne venete, incriminazioni
Mastelloni) e triangolazione con corpus: doppio canale armamenti BR,
lodo Moro, Hyperion (prosciolto 1990), eco di metodo Nasco. Registro
verifiche aggiornato a voce 40.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2231,6 +2231,51 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>ARSENALE SARDO delle Brigate Rosse (Lula, Monte Albo-Monte Pitzinnu, febbraio 1982) - ricognizione delle armi e TRIANGOLAZIONE con il corpus (canale OLP, lodo Moro, Hyperion, Barbagia Rossa)</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>repertorio (foglio di servizio - ricognizione e triangolazione)</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>FATTO (A): 23-27.2.1982, campagne di Lula (NU) tra Monte Albo e Monte Pitzinnu: deposito BR scoperto su indicazione del pentito Savasta; custodia di Barbagia Rossa; possibile destinazione l'assalto a Badu 'e Carros (B). INVENTARIO di fonte sarda: cinque razzi per bazooka USA, UN missile anticarro sovietico, due missili ARIA-TERRA francesi, trenta chili di plastico, otto bombe a mano USA, sei mitra Sterling inglesi, un centinaio di cartucce. Discrepanze del paragrafo circolante in inglese dichiarate (plurali amplificati, 'aria-aria', 'centinaia'). FILIERA (A): viaggio del Papago (Moretti, agosto 1979, Numana-Cipro-Libano) e consegne OLP su spiagge venete (settembre 1979: Sterling, lanciarazzi, esplosivi); incriminati da Mastelloni Abu Ayad e Abu Jihad; retroterra del lodo Moro (B).</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE: (1) doppio canale degli armamenti BR - Skorpion di Moro dal mercato interno (Sanremo 1971, voce 35), arsenale di Lula dal canale OLP: due filiere parallele che si confermano; (2) fronte carcerario: colonna sarda nata per Asinara/Badu 'e Carros; (3) lodo Moro = quadro mediterraneo gia' censito nel corpus; (4) Hyperion/Superclan come snodo ambiguo alla maniera di Aginter (paragone METODOLOGICO); (5) il catalogo 'internazionalista' delle armi dimostra il bazar OLP, NON una regia sovietica.</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Fragilita' dichiarate: filone Hyperion chiuso con PROSCIOGLIMENTO GENERALE 1990 (imputati anche i generali Lugaresi, Notarnicola, Grassini) - incriminato NON e' condannato, resta allegazione istruttoria (C); tesi della catena di comando Mosca-BR = tesi pubblicistica alla Claire Sterling, mai accertata (C); identita' pezzo-per-pezzo carico Papago-arsenale Lula non cristallizzata in sentenza (B); pista sarda-bolognese del 'passaporto di Aritzo' = C; eco di metodo coi depositi Nasco/Gladio senza equivalenza. Convergenza di milieu diverso da catena di comando. INCROCI: voci 35-36-39 (balistica Moro), registri D7 e mediorientali. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>RICOGNIZIONE E TRIANGOLAZIONE CERTIFICATE (con proscioglimenti e tesi di parte dichiarati). Domini: D7, D3.</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>repertorio/ITALIA_NERA_ARSENALE_SARDO_TRIANGOLAZIONE.xlsx (Excel di servizio, 6 fogli)</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Triangolazione NASCO-Gladio e catena Skorpion col corpus (voce 41)
Verifica preliminare dei due testi ricevuti e doppio aggancio al
corpus: impianto NASCO confermato (139 depositi, Aurisina 1972,
127 recuperati, cerniera Peteano-Casson), testo Skorpion corretto
(due armi distinte, covo di via Dogali giugno 1988, matricola 5075
non riscontrata, promozioni indebite declassate). Specularita' dei
depositi con l'arsenale di Lula e circolarita' del mercato nero
delle armi. Registro verifiche aggiornato a voce 41.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2276,6 +2276,51 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE NASCO di Gladio + catena della Skorpion (due testi ricevuti) con il corpus - verifica preliminare dei testi e doppio aggancio (voci 35-36, 39-40, strategia della tensione)</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica + repertorio (verifica di testi ricevuti e triangolazione)</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>NASCO (impianto CONFERMATO): 139 depositi e 622 gladiatori (dati Andreotti 1990); protocollo SIFAR-CIA 26.11.1956 (De Lorenzo); CAG di Capo Marrargiu; scoperta casuale di Aurisina (24.2.1972) e recupero 1972-73 di 127 NASCO su 139 - DODICI mai recuperati; Peteano a pochi km tre mesi dopo, sospetto Casson su esplosivo/detonatore (istruttorio, mai in sentenza); Serravalle imputato di falso su Aurisina. SKORPION (testo CORRETTO in tre punti): DUE armi distinte, non una - la Skorpion di Morucci (Roma 1979) indicata dalle perizie come arma di Moro, e la ex Jimmy Fontana (Sanremo 1971) sequestrata in VIA DOGALI (Milano, 15-18.6.1988, non 'via Griffini/ottobre') e legata ad Acca Larentia 1978, Tarantelli 1985, Conti 1986, Ruffilli 1988; 'matricola 5075' NON riscontrata; Palma, Tartaglione e Hunt promossi indebitamente a Skorpion (arma non modellizzata: C).</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE: (1) specularita' dei depositi - NASCO di Gladio vs arsenale BR di Lula (voce 40): stessa tecnica, finalita' opposte, Sardegna su entrambi i fronti (Capo Marrargiu / Lula); eco di metodo formalizzato; (2) doppio canale armamenti BR confermato: nessuna delle due Skorpion proviene dai NASCO - il sospetto 'armi NATO alle BR' resta senza riscontro in questa catena; (3) Peteano come cerniera giudiziaria: dal processo Casson alla rivelazione di Gladio (1990); (4) la Skorpion di via Dogali attraversa i fronti opposti (Acca Larentia MSI - omicidi BR-PCC): il singolo reperto che meglio dimostra la circolarita' del mercato nero delle armi; (5) ipotesi FARL su Hunt = quadro mediterraneo del lodo Moro (C).</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Fragilita' e correzioni dichiarate: la voce 35 registrava in B l'identita' 'Skorpion via Dogali = arma di Moro' - questa triangolazione la DECLASSA a favore della ricostruzione a due armi (perizie d'archivio unica via di chiusura); tesi 'esplosivi NASCO nelle stragi' = C senza promozione (i dodici NASCO mancanti sono dato aperto, non prova); Rocca: morte archiviata come suicidio, tesi omicidio = C; attribuzioni Marras/de Lellis/Polgar e dettagli (radio 'Angora', prede belliche, sommergibili) = C non riscontrati; errori materiali dei testi corretti (via Montalcini, via Dogali, date recupero NASCO). Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE CERTIFICATA CON VERIFICA PRELIMINARE DEI TESTI (correzioni e declassamenti dichiarati). Domini: D7, D3, D4.</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>repertorio/ITALIA_NERA_NASCO_SKORPION_TRIANGOLAZIONE.xlsx (Excel di servizio, 7 fogli)</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Censimento capillare NASCO, arsenali BR e Superclan (voce 42)
Mappa regionale completa dei 139 NASCO (127 recuperati, dodici
irrisolti con due siti localizzati), dotazioni da atti; nove
arsenali/covi BR censiti con inventari (da via Gradoli a via
Dogali); Superclan: assenza di arsenali fisici dichiarata come
esito - solo intermediazione contestata e prosciolta. Incrocio
Sterling/Energa tra via Fracchia e Lula. Registro verifiche
aggiornato a voce 42.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2321,6 +2321,51 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>CENSIMENTO CAPILLARE: i 139 NASCO di Gladio (mappa regionale e dotazioni), nove arsenali/covi BR con inventari, 'arsenali del Superclan' (esito: assenza dichiarata)</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>repertorio (censimento dei tre sistemi di arsenali clandestini)</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>NASCO (A): mappa regionale completa - FVG cento, Lombardia undici, Veneto sette, Piemonte sette, Trentino cinque, Liguria quattro, Emilia-Romagna due, Puglia due, Campania uno = 139; interrati dal 1963; recupero post-Aurisina chiuso nel 1973: 127 recuperati, DODICI mai recuperati, di cui due localizzati in rete (cappella del cimitero di Mariano del Friuli: 2 contenitori metallici + 3 plastica; Santa Petronilla di San Vito al Tagliamento: 2+2); dotazione tipo da atti (armi portatili, munizioni, esplosivi, bombe a mano, fucili di precisione, radio). ARSENALI BR (nove siti censiti con inventario): Robbiano di Mediglia 1974, Cascina Spiotta 1975, via Gradoli 1978 (Sten, Reck, Beretta 6,35/1941, cal.22 950, fucile a pompa USA, 17 candelotti dinamite, 75 detonatori), via Monte Nevoso 1978 (cinque armi corte, 770 g polvere da mina, due bombe a mano + doppio fondo 1990 con fucile e 40 detonatori), viale Giulio Cesare 1979 (arsenale Morucci con la Skorpion di Moro), via Fracchia 1980 (cinque pistole, DUE STERLING, fucile Franchi, 2000 cartucce, DUE ENERGA, due mine anticarro, plastico), via Silvani 1980 (PPK/S 47/18), Lula 1982 (voce 40), via Dogali 1988 (Skorpion ex Fontana).</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>SUPERCLAN: NESSUN arsenale fisico mai sequestrato o censito - solo presunta INTERMEDIAZIONE di armi OLP (Galati, Savasta; incriminazioni Mastelloni 1982) con proscioglimento 1990: il Superclan non aggiunge siti alla mappa, aggiunge (in ipotesi mai giudicata) una regia sul flusso. INCROCIO CENTRALE: Sterling ed Energa compaiono sia in via Fracchia sia a Lula = la tipologia del canale OLP si distribuisce su colonne del nord e deposito sardo. NASCO e BR: nessun travaso accertato tra le due filiere.</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Limiti dichiarati: elenco integrale dei 139 NASCO con distinte di carico negli atti (Commissione stragi/doc. Andreotti), non in rete - qui mappa regionale e due dei dodici irrisolti; inventari di Robbiano e Cascina Spiotta non modellizzati in rete (giallo); censimento BR = covi-arsenale maggiori documentati, non le basi minori; tracciabilita' pezzo-per-pezzo del canale OLP solo dagli atti (C). INCROCI: voci 39-41. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>CENSIMENTO CERTIFICATO CON LACUNE D'ARCHIVIO DICHIARATE. Domini: D7, D3, D4.</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>repertorio/ITALIA_NERA_CENSIMENTO_NASCO_ARSENALI_BR_SUPERCLAN.xlsx (Excel di servizio, 7 fogli)</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Censimento arsenali NAR, Avanguardia Nazionale e Banda della Magliana (voce 43)
Gemello della voce 42 sul fronte nero-criminale: arsenale-madre della
Magliana nei sotterranei del Ministero della Sanita' (via Liszt 1981,
con le Gevelot del tipo Pecorelli e le armi condivise coi NAR), covo
NAR di via Alessandria (1979, nodo Amato-Straullu), Avanguardia
Nazionale come flusso senza siti (Roma-Reggio, istruttore OAS,
Camerino). Triangolazione: lo Stato come deposito, rovescio dei NASCO.
Registro verifiche aggiornato a voce 43.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2366,6 +2366,51 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>CENSIMENTO ARSENALI del fronte nero-criminale romano: NAR, Avanguardia Nazionale, Banda della Magliana (gemello della voce 42)</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>repertorio (censimento arsenali - fronte nero-criminale)</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>MAGLIANA (A): arsenale-madre nei sotterranei del MINISTERO DELLA SANITA' (via Franz Liszt 34, EUR), scoperto il 27.11.1981: custode l'usciere Biagio Alesse (un milione di lire al mese, intermediario la guardia giurata Alvaro Pompili); inventario: diciannove pistole/revolver, Beretta M12, MAB 38, Sten, altri mitra, cartucce, bombe a mano, esplosivi, materiale per travisamento. REPERTO-CHIAVE: quattro proiettili GEVELOT dello stesso raro tipo di quelli che uccisero Pecorelli (ponte materiale con la voce 39; assoluzioni definitive di Perugia dichiarate). Arsenale CONDIVISO coi NAR (armi di entrambi). NAR (A): via Alessandria (dic. 1979: undici pistole, granate, esplosivi, divise da carabiniere) - crocevia di servizi e neofascisti legato agli omicidi Amato e Straullu, con ipotesi di depistaggio fino a Bologna (C); Acilia (granate da via Alessandria); via Decio Mure (Vale, giallo). AN: NESSUN arsenale unitario - flusso di armi/esplosivi/timer Roma-Reggio Calabria sotto supervisione Delle Chiaie, istruttore ex OAS in via Michele Amari (aggancio Aginter/OAS del corpus), arsenale-provocazione di Camerino (Fachini-SID, C), archivio segreto Delle Chiaie (2021, cartaceo).</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE: (1) lo Stato come deposito - rovescio speculare dei NASCO (voce 42): la' lo Stato interrava armi nel territorio, qui il crimine interrava armi dentro un ministero; (2) la cerniera nera-criminale (NAR-Magliana) = logistica comune, matrice del Mondo di mezzo; (3) ponte Gevelot-Pecorelli documentato come reperto, non come responsabilita'; (4) l'istruttore OAS = eco diretto delle monografie Aginter del corpus; (5) morfologia comparata: BR arsenali propri, fronte nero arsenali condivisi e flussi senza siti.</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Fragilita' dichiarate: assoluzioni definitive nel processo Pecorelli (il reperto resta reperto); Camerino come provocazione = ricostruzione istruttoria (C); nesso via Alessandria-Bologna = C senza promozione; inventari dei depositi minori (Magliana, via Decio Mure) non modellizzati in rete - direzione d'archivio. INCROCI: voci 39, 41, 42; monografie Aginter; registro strategia della tensione. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>CENSIMENTO CERTIFICATO (fronte nero-criminale; assoluzioni e ipotesi dichiarate). Domini: D7, D4, D6.</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>repertorio/ITALIA_NERA_ARSENALI_NAR_AN_MAGLIANA.xlsx (Excel di servizio, 7 fogli)</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Triangolazione terminale a cento blocchi sugli arsenali (voce 44)
Matrice di confronto a cento blocchi tra i NASCO e tutti gli arsenali
censiti (BR, NAR, AN, Magliana, Superclan), estesa a Rosa dei Venti/NDS,
MAR di Fumagalli e al sistema-radice delle armi partigiane occultate.
Verdetto: specularita' di metodo, geografia e code irrisolte PROVATE;
affinita' di radice e materiale PROVATE (bacino della guerra civile,
standard NATO); travaso Stato-eversione e regia unica NON provati e
dichiarati tali. Registro verifiche aggiornato a voce 44.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2411,6 +2411,51 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE TERMINALE A CENTO BLOCCHI: NASCO contro/accanto a tutti gli arsenali censiti (BR, NAR, AN, Magliana, Superclan) + due sistemi nuovi (Rosa dei Venti/NDS, MAR di Fumagalli) + il sistema-radice delle armi partigiane occultate</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>repertorio (matrice di confronto a cento blocchi)</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Mandato ('fare di tutto perche' emerga natura speculare o affine') eseguito come OBBLIGO DI PROFONDITA', non di esito. VERDETTO: (1) SPECULARITA' DI METODO PROVATA (A) - interramento, compartimentazione, custodi fiduciari remunerati, travisamento, patti internazionali segreti (SIFAR-CIA 1956 / BR-OLP 1979), organi ristretti con le mappe; (2) AFFINITA' DI MATERIALE PROVATA (A) - stesso bacino di residuati della guerra civile 1943-45 (Sten, MAB, TZ-45, FNAB-43: quest'ultima da via Fani all'Algeria), stessi standard NATO (Sterling, Energa, 9 Para), stessi plastici e detonatori; (3) AFFINITA' DI RADICE PROVATA (A/B) - tutte le reti discendono dalla guerra civile e dalle sue armi occultate (caso Val di Susa); (4) SPECULARITA' GEOGRAFICA PROVATA (A) - Sardegna (Capo Marrargiu/Lula), Nord-Est (100 NASCO/spiagge OLP), Alpi (Trentino/Valtellina MAR), Roma armeria diffusa, Parigi doppia centrale (CPC/Hyperion); (5) SPECULARITA' DELLE CODE PROVATA (A) - 12 NASCO, PPK di Moro, pistola di Pecorelli, reperti spariti, matricole abrase.</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>NUOVI SISTEMI CENSITI IN CAMPAGNA: Rosa dei Venti/Nuclei per la Difesa dello Stato (dispositivo parallelo dal 1964, atti Tamburino, inchiesta avocata dalla Cassazione 1978) e MAR di Fumagalli (ex partigiani bianchi, Valtellina, esplosivi sequestrati marzo 1974, referenti indicati Sogno/Taviani) = la 'matrioska' delle reti parallele, provata come PLURALITA' (B), non come catena unica. TRAVASO eversione-crimine PROVATO (arsenale condiviso NAR-Magliana). Il chiasmo di sintesi: lo Stato-seminatore (NASCO nel territorio) contro lo Stato-contenitore (la Magliana nel ministero).</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>NON PROVATO E DICHIARATO: travaso fisico Stato-eversione (unico ponte ipotizzato Peteano, istruttorio, C); regia unica dei due fronti (tesi sovietica alla Sterling e tesi dello Stato-stragista integrale: entrambe C). La specularita' e' un fatto morfologico certificato; l'identita' operativa sarebbe una tesi e resta tale. Metodo: cento blocchi alimentati dalle voci 35-43 + campagna nuova (Rosa dei Venti, MAR, residuati, FNAB-43). INCROCI: voci 35-43, monografie Aginter (istruttori OAS), registro strategia della tensione. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE TERMINALE CERTIFICATA (specularita' e affinita' emerse ai gradi dichiarati; identita' non promossa). Domini: D7, D4, D3.</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>repertorio/ITALIA_NERA_TRIANGOLAZIONE_CENTO_BLOCCHI_ARSENALI.xlsx (Excel di servizio, 4 fogli, 100 blocchi)</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Triangolazione a 250 blocchi della matrice arsenali coi casi del corpus (voce 45)
Duecentocinquanta blocchi = venticinque casi principali del corpus x
dieci assi, con Excel di servizio e DOCX di prosa. Verdetto trasversale:
specularita' e affinita' dei sistemi certificate su metodo, materiale,
radice (guerra civile 1943-45), geografia e code irrisolte; travaso
eversione-crimine provato; travaso Stato-eversione e regia unica non
provati. Vertice Putin: convergenza sistemica euroasiatica, non catena
di comando. Registro verifiche aggiornato a voce 45.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2456,6 +2456,51 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE della matrice a cento blocchi (voce 44) con i VENTICINQUE CASI PRINCIPALI del corpus - 250 blocchi mirati - Excel + DOCX</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica (DOCX di prosa) + repertorio (Excel a 250 blocchi)</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Struttura: 250 blocchi = 25 casi x 10 assi (metodo/logistica, materiale bellico, radice storica, geografia, uomini/custodi/formatori, regia/patti, code irrisolte, esito giudiziario, travaso/cerniera, verdetto del caso). CASI: esecuzione Moro, via Fani, trittico PPK/M34, Arsenale Sardo, NASCO, catena Skorpion, arsenali BR, Superclan/Hyperion, NAR, Avanguardia Nazionale, Magliana, Rosa dei Venti/NDS, MAR Fumagalli, matrice cento blocchi, piazza Fontana, Bologna, piazza della Loggia, Peteano, Aginter/Guerin-Serac, Delle Chiaie/Condor, apartheid Sudafrica-Namibia, Brighton Beach/Bratva, Cinque Famiglie, cluster Trump, Putin. Campagna di ricerca nuova su: esplosivo di Bologna (TNT+T4 da residuato bellico), gelignite di piazza Fontana (timer Junghans-Diehl, candelotti di Trieste-Gorizia), Aginter (60% personale ex OAS), dimensione armiera della Bratva (elicotteri Armata Rossa, Fainberg).</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>VERDETTO TRASVERSALE ai 250 blocchi: la natura SPECULARE e AFFINE dei sistemi e' EMERSA E CERTIFICATA (A) su cinque dimensioni - metodo dell'occultamento, materiale/standard (residuati 1943-45 + NATO), radice nella guerra civile, geografia (Sardegna, Nord-Est, Alpi, Roma, Parigi), simmetria delle code irrisolte (armi mai ritrovate, reperti spariti). Travaso eversione-crimine PROVATO (arsenale condiviso NAR-Magliana). Il vertice Putin: la galassia Aginter/apartheid NON converge sul Cremlino (antipode atlantista); l'unico ponte reale e' la spina euroasiatica del crimine organizzato = convergenza sistemica, non catena di comando personale.</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>NON PROVATO E DICHIARATO: travaso fisico Stato-eversione (unico appiglio Peteano, istruttorio, C); regia unica dei due fronti (tesi sovietica alla Sterling e Stato-stragista integrale: C); Putin-regista (C). La specularita' e' un fatto morfologico certificato; l'identita' operativa resta tesi. Ogni blocco col proprio grado Savona. INCROCI: voci 35-44 e i registri analitici del corpus (Aginter, guerra fredda, Sudafrica-Sudamerica, censimento criminalita', Putin). Vincolo fonti rispettato (no Grokipedia, no il manifesto ne' il manifesto in rete).</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE TERTMINALE CERTIFICATA (250 blocchi; specularita'/affinita' emerse ai gradi dichiarati; identita' e regia unica non promosse). Domini: D7, D4, D3, D1, D2.</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica/ITALIA_NERA_TRIANGOLAZIONE_250_BLOCCHI_CORPUS.docx + repertorio/ITALIA_NERA_TRIANGOLAZIONE_250_BLOCCHI_CORPUS.xlsx</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Triangolazione dei 25 personaggi centrali per numero di nodi (voce 46)
Duecentocinquanta blocchi = 25 personaggi (classificati per frequenza
di menzione come proxy dei nodi) x 10 assi, con Excel e DOCX. Verdetto:
struttura bicefala del corpus - blocco egemone nero-atlantista antipode
di Putin, blocco euroasiatico attorno a Putin, collegati solo dal ponte
dottrinale Thiriart-Dugin e dalla spina crimine-energia Mogilevich-
Firtash-Kovalchuk. Convergenza sistemica certificata, catena di comando
unica non provata. Registro verifiche aggiornato a voce 46.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2501,6 +2501,51 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE dei PRIMI VENTICINQUE PERSONAGGI del corpus PER NUMERO DI NODI con l'intero corpus - 250 blocchi mirati - Excel + DOCX</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica (DOCX di prosa) + repertorio (Excel a 250 blocchi)</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICA (proxy = frequenza di menzione su 95 file, &gt;4 milioni di caratteri; cautela dichiarata su omonimie/locuzioni): 1 Guerin-Serac (615), 2 Delle Chiaie (362), 3 Putin (176), 4 P.W. Botha (115), 5 Skorzeny (114), 6 Kissinger (107), 7 Gelli (101), 8 Aldo Moro (91, gonfiato da 'lodo/commissione Moro'), 9 Dugin (79), 10 Pinochet (75), 11 Vinciguerra (71), 12 Giannettini (68), 13 Klaus Barbie (59), 14 Thiriart (59), 15 Mogilevich (50), 16 Borghese (46), 17 Robert Leroy (38), 18 Vorster (35), 19 Michael Cohen (35), 20 Carminati (33), 21 Andreotti (29), 22 Williamson (29), 23 Khodorkovsky (27), 24 Firtash (25), 25 Kovalchuk (23). STRUTTURA: 250 blocchi = 25 personaggi x 10 assi (dominio, rete, geografia, funzione, cerniera con altri nodi, rapporto Stato/servizi, esito giudiziario, aggancio Putin/euroasia, code irrisolte, verdetto del nodo).</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>VERDETTO TRASVERSALE: il corpus e' BICEFALO. Blocco EGEMONE nero-atlantista (Guerin-Serac, Delle Chiaie, Botha, Skorzeny, Kissinger, Gelli, Pinochet, Vorster, Barbie, Williamson, Leroy, Borghese, Vinciguerra, Giannettini, Carminati, Andreotti) che NON converge su Putin ma ne e' l'ANTIPODE di guerra fredda. Blocco EUROASIATICO (Putin, Dugin, Thiriart, Mogilevich, Firtash, Kovalchuk, Khodorkovsky, Cohen). I due mondi si toccano SOLO in due punti: (a) ponte DOTTRINALE Thiriart-&gt;Dugin; (b) SPINA crimine-energia Mogilevich-Firtash-Kovalchuk. Kovalchuk = aggancio piu' diretto (cerchia Ozero); Khodorkovsky converge IN NEGATIVO (oligarca espulso).</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Fragilita' dichiarate: la classifica e' ordinamento di centralita' (frequenza-proxy), NON conteggio notarile dei nodi - omonimie e locuzioni ('lodo Moro', 'Cohen') dichiarate caso per caso; su viventi (Putin, Cohen, Khodorkovsky, Firtash, Kovalchuk) massimo rigore; tesi 'Putin-regista', influenza Dugin sul Cremlino, caso Palme/Williamson = C. Convergenza sistemica e di milieu certificata; catena di comando unica NON provata. INCROCI: voci 35-45 e i registri analitici dei nodi (Aginter, apartheid, D1 criminalita', sotto-hub russi). Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE DEI NODI-PERSONA CERTIFICATA (250 blocchi; struttura bicefala; convergenza certificata, catena unica non promossa). Domini: D7, D3, D2, D6, D1, D8.</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica/ITALIA_NERA_TRIANGOLAZIONE_250_BLOCCHI_PERSONAGGI.docx + repertorio/ITALIA_NERA_TRIANGOLAZIONE_250_BLOCCHI_PERSONAGGI.xlsx</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Registro analitico dei nodi: versione integrale e rinnovata (voce 47)
Consolidamento di tutti i registri-nodi del corpus (Aginter/apartheid,
censimento criminalita' D1, integrazione e archi, sotto-hub euroasiatici,
hub P2) piu' trenta nodi nuovi dalle voci 35-46 (balistica Moro, arsenali,
reti parallele, stragi, dorsale euroasiatica): 260 nodi dedotti su nove
domini, con indice per dominio, dieci grandi hub e sinapsi principali.
Excel a cinque fogli + DOCX di prosa. Registro verifiche a voce 47.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2546,6 +2546,51 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>REGISTRO ANALITICO DEI NODI - versione INTEGRALE e RINNOVATA: consolidamento di tutti i registri-nodi + i nodi nuovi delle voci 35-46 - Excel + DOCX</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (DOCX) + repertorio (Excel del registro integrale)</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>260 NODI consolidati per estrazione automatica dai registri-fonte (Aginter/apartheid integrazione+approfondimento, censimento criminalita' D1, integrazione e archi, sotto-hub euroasiatici gas/media/riciclaggio/EUB/Khodorkovsky, hub P2), deduplicazione per nome con unione dei domini, e aggiunta di 30 nodi nuovi dalle voci 35-46 (PPK e Skorpion di Moro, Jimmy Fontana, Walter Rossi, via Silvani; arsenale di Lula, Barbagia Rossa, Papago, lodo Moro; NASCO, Aurisina, Capo Marrargiu; arsenale del Ministero della Sanita', Alesse, via Alessandria; Rosa dei Venti/NDS, Spiazzi, MAR, Fumagalli, FNAB-43; quattro stragi; Brighton Beach, Ivankov, Fainberg, cluster Trump/Cohn/Sater). Distribuzione: D1=67, D7=48, D2=43, D6=34, D3=27, D4=16, D9=12, D10=9, D8=4.</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>STRUTTURA a 5 fogli: quadro; registro integrale (260 nodi con dominio primario, tutti i domini, descrizione, registro di provenienza); indice per dominio con conteggi; dieci grandi hub per centralita' (Guerin-Serac, Delle Chiaie, Putin, Gelli, Botha/Vorster, Mogilevich, Carminati, Moro, Thiriart-&gt;Dugin, Kovalchuk/Firtash); sinapsi principali con grado (compreso l'arco NEGATIVO galassia Aginter/apartheid -&gt; Putin = nessuna convergenza, antipode). Il registro integrale e' la vista d'insieme che sussume i registri parziali (che restano fonti di dettaglio).</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: registro DESCRITTIVO dei nodi e degli archi; la gradazione probatoria dei singoli fatti resta nei registri analitici di dominio e nel registro delle verifiche (voci 35-46). Massimo rigore sui viventi (Putin, Cohen, Firtash, Kovalchuk, Khodorkovsky); nessuna convergenza sistemica promossa a catena di comando personale. Correzione tecnica: i nodi del censimento D1 (col localita') riclassificati correttamente sotto D1 (zero nodi non classificati). INCROCI: tutti i registri-nodi del corpus e le voci 35-46. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>REGISTRO INTEGRALE DEI NODI GENERATO E CERTIFICATO (260 nodi, 9 domini, 10 hub, sinapsi principali). Domini: tutti (D1-D10).</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/ITALIA_NERA_REGISTRO_ANALITICO_NODI_INTEGRALE.docx + repertorio/ITALIA_NERA_REGISTRO_ANALITICO_NODI_INTEGRALE.xlsx</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monografia dei grandi hub, parte prima: nodi, sinapsi, ponti e casi (voce 48)
Primo DOCX della serie sui personaggi ed entita' con piu' nodi
certificati: i dieci grandi hub del corpus spiegati per filo e per
segno (Guerin-Serac/Aginter, Delle Chiaie, Putin, Gelli/P2, Stato
apartheid Botha-Vorster, Mogilevich, Carminati, Aldo Moro, ponte
Thiriart-Dugin, coppia Kovalchuk-Firtash), con nodi, sinapsi, ponti,
casi ed evidenze. Struttura bicefala e tre nature di legame dichiarate.
Registro verifiche aggiornato a voce 48.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2591,6 +2591,51 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>MONOGRAFIA dei GRANDI HUB (parte prima): i dieci nodi a piu' alta centralita' del corpus spiegati per filo e per segno - nodi, sinapsi, ponti, casi ed evidenze - DOCX pubblicato</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (DOCX monografico dell'opera)</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Primo DOCX della serie sui personaggi/entita' con piu' nodi certificati (criterio: voci 46-47). Tratta i DIECI GRANDI HUB: (1) Yves Guerin-Serac/Aginter Press (nodo-madre; OAS 60%; raid 1974; assassinii Mondlane 1969, Cabral 1973); (2) Stefano Delle Chiaie (AN, Aginter, Condor, golpe Bolivia 1980; assolto piazza Fontana); (3) Vladimir Putin (vertice euroasiatico; siloviki/Ozero; tre sinapsi Kovalchuk/Firtash-Mogilevich/Dugin; massimo rigore); (4) Licio Gelli/P2 (hub eversione-Stato-finanza; mandante Bologna nelle sentenze; liste Castiglion Fibocchi); (5) Stato dell'apartheid Botha/Vorster (entita'; BOSS/NIS; Williamson; omicidi First 1982, September 1988, Lubowski 1989; amnistie TRC); (6) Semyon Mogilevich (architetto crimine euroasiatico; Ivankov/Brighton Beach 1992; RosUkrEnergo; BoNY); (7) Massimo Carminati (cerniera NAR-Magliana; arsenale ministero 27.11.1981; Gevelot-Pecorelli; assoluzioni); (8) Aldo Moro (vittima baricentrica; via Fani 91 bossoli e FNAB-43; esecuzione PPK+Skorpion; PPK mai ritrovata); (9) ponte dottrinale Thiriart-&gt;Dugin (Jeune Europe 1962-69; eurasiatismo); (10) coppia finanziaria Kovalchuk-Firtash (Bank Rossiya/Ozero 1996; sanzioni 2014; RUE/Gazprom).</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>STRUTTURA BICEFALA esplicitata: 7 hub nel blocco nero-atlantista (antipode di Putin), 3 nel blocco euroasiatico, 1 ponte dottrinale di cerniera. Tre nature di legame distinte e dichiarate: (a) sinapsi operative accertate (Serac-Leroy in Aginter; NAR-Magliana nell'arsenale = travaso PROVATO); (b) ponti di metodo/idee (eco Aginter nelle stragi; Thiriart-&gt;Dugin = convergenza, non committenza); (c) l'ARCO NEGATIVO: la galassia Aginter/apartheid NON converge su Putin (antipode). Specularita'/affinita' = fatto morfologico certificato; identita' operativa = tesi non promossa.</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: documento narrativo-monografico che rende in prosa le evidenze gia' gradate nei registri (voci 35-47); massimo rigore sui viventi (Putin, Kovalchuk, Firtash); assoluzioni dichiarate (Delle Chiaie piazza Fontana; Carminati/Pecorelli); mandato Bologna di Gelli come accertamento raggiunto. 'Parte prima' = seguiranno monografie sugli hub successivi in graduatoria. INCROCI: voci 35-47; registro analitico integrale dei nodi. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>MONOGRAFIA DEI GRANDI HUB (PARTE PRIMA) PUBBLICATA. Domini: D7, D3, D2, D6, D4, D1.</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/ITALIA_NERA_MONOGRAFIA_GRANDI_HUB_PARTE_PRIMA.docx</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Opera monumentale, Fase I: la centrale e la radice (Aginter Press) (voce 49)
Prima delle cinque Fasi che riordinano l'intero corpus in 50 capitoli e
250 nodi/ponti certificati. Fase I: 10 capitoli, 50 nodi/ponti (I.1-I.50)
sulla galassia nera internazionale - Aginter Press, Guerin-Serac, la
matrice OAS, Delle Chiaie, Ordine Nuovo, i servizi di copertura,
l'internazionale reazionaria, la dottrina religiosa, le operazioni
africane, con tre triangolazioni finali e l'arco negativo galassia-Putin.
Stile accademico, numeri in cifre arabe (generatore dedicato). Registro
verifiche a voce 49.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2636,6 +2636,51 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>OPERA MONUMENTALE in 5 Fasi / 50 Capitoli / 250 nodi-ponti - FASE I: 'La centrale e la radice: Aginter Press e la galassia nera internazionale' - DOCX (stile accademico, cifre arabe)</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (DOCX della Fase I dell'opera monumentale)</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Prima delle cinque Fasi dell'opera che riordina l'intero corpus. FASE I, 10 capitoli, 50 nodi/ponti certificati (numerati I.1-I.50): Aginter Press e Guerin-Serac (nodo-madre), Robert Leroy, raid 1974; dottrina (Notre action politique 1968-69, guerre revolutionnaire, Ordre et Tradition, OACI); matrice OAS/algerina (11e Choc, istruttore di via Michele Amari); Delle Chiaie e Avanguardia Nazionale; Ordine Nuovo (Rauti, Zorzi, Maggi); servizi (PIDE/DGS, liaison CIA-PIDE 1957, rapporto SDCI, BND/Gehlen); internazionale reazionaria (Le Cercle, Crozier, Damman, Thiriart-&gt;Dugin); dottrina religiosa (Cite Catholique, Giannettini, convegno Pollio 1965); operazioni africane (Mondlane 1969, Cabral 1973, ponte verso apartheid/Williamson); 3 triangolazioni finali + arco negativo galassia-Putin + appendice analitica sulle evidenze.</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Requisiti dell'autore rispettati: stile accademico (Crusca/Treccani); NUMERI IN CIFRE ARABE (deroga esplicita al guardiano anti-cifre, generatore dedicato gen_docx_cifre.py che mantiene A4/Times New Roman 12/giustificato); triangolazioni incrociate tra nodi e ponti diversi; struttura 5 Fasi/50 Capitoli/250 nodi-ponti (questa e' la Fase I). Statuto Savona applicato in prosa (certo/probabile/candidato/negativo); tesi bicefala del corpus e ponte negativo galassia nera&lt;-&gt;Putin come architrave.</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>NOTA DI LUNGHEZZA DICHIARATA: la Fase I e' completa nella struttura (10 capitoli, 50 nodi/ponti, appendice) ma consta di circa 8.750 parole, contro il bersaglio di +/-20.000 parole per Fase indicato dall'autore. La lunghezza piena e' raggiungibile con ulteriore espansione capitolo per capitolo (piu' contesto storico-biografico ed evidenziale); in attesa di disposizione dell'autore, che ha chiesto di fermarsi dopo ogni Fase. Vincolo fonti rispettato (no Grokipedia, no il manifesto). Si procede una Fase per volta.</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>FASE I DELL'OPERA MONUMENTALE GENERATA (struttura completa; lunghezza da confermare/espandere). Domini: D7, D3, D10, D2.</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/ITALIA_NERA_OPERA_MONUMENTALE_FASE_I.docx</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atto di ricezione: 21 documenti d'autore nel corpus (Moro Fase Settima, Tavola Unica) (voce 50)
Ingestione nel corpus/opera di 21 file nuovi (deduplicati): la serie
'Aldo Moro - Il Registro dei Cinquantacinque Giorni', Fase Settima, con
dieci appendici (seconda-dodicesima, verifica genealogica delle fonti e
apparato dell'Indice generale atti X legislatura); la Prima Sessione
Esecutiva della Tavola Unica (Sezione Metafisica); la Tutta la Verita'
Triangolazione (matrice probatoria); piu' materiali di ricerca su
diaspora nazista, Citta' del Capo e arsenale Magliana. Registro
verifiche a voce 50. Mancano dalla serie le appendici prima e settima.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2681,6 +2681,51 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>ATTO DI RICEZIONE: ingresso nel corpus di 21 documenti d'autore nuovi - la linea 'ALDO MORO - Il Registro dei Cinquantacinque Giorni' (Fase Settima), la Tavola Unica, la Tutta la Verita' e materiali di ricerca</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (ingesti con nome pulito, senza prefisso UUID)</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Ricevuti e collocati in corpus/opera 21 file (deduplicati per contenuto; saltati 20 gia' presenti e 7 doppioni identici). NUCLEO PRINCIPALE - serie 'ALDO MORO - IL REGISTRO DEI CINQUANTACINQUE GIORNI' (autore Luigi De Michele, agosto 2026): dieci Appendici alla FASE SETTIMA (seconda, terza, quarta, quinta, sesta, ottava, nona, decima, undicesima, dodicesima) - documenti di verifica genealogica delle fonti, sull'apparato dell'Indice generale atti della X legislatura (Commissione Moro 2, 102 sedute), che NON modificano i 70 Capitoli dell'opera Moro ma ne raffinano l'apparato probatorio. Inoltre: ITALIA_NERA_PRIMA_SESSIONE_ESECUTIVA_TAVOLA_UNICA (Sezione Metafisica, Religiosa ed Esoterica; verbale in 20 blocchi; chiusura L38, avanzamento L36-L37, voci L39-L43); Opera_Aldo_Moro_Tutta_la_Verita_Triangolazione (consolidamento della matrice probatoria: genealogia delle fonti, fonte derivata, indipendenza, lacuna, causalita', ponte documentale, autore materiale).</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Materiali di ricerca annessi: Diaspora_Nazista_PostBellica_Ricerca_Approfondita_2 (3 MB); Come_i_simzia_1 (simpatizzanti nazisti a Citta' del Capo, Robey Leibbrandt - materiale asse Sudafrica/diaspora nazista, Fase II); Clandestine_Arms_Caches_and_Subversive_Networks (fonte diretta sull'arsenale della Magliana in via Liszt - riscontro della voce 43); cinque registri analitici di sessione in versione senza suffisso (Aginter/Sudafrica-Sudamerica, Guerra Fredda, sessione 2 agosto, Aginter-Sunniti, PayPal-Apartheid, Asse Asiatico-Pacifico).</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: ATTO DI RICEZIONE, non verifica: i documenti entrano come fonti/opere d'autore, conservate cumulativamente (nulla si cancella). MANCANTI dalla serie Moro: appendice PRIMA e appendice SETTIMA (non presenti nel lotto caricato) - da richiedere all'autore per completare la Fase Settima. La linea 'Registro dei Cinquantacinque Giorni' (70 Capitoli + Fase Settima) e' opera parallela dell'autore, di cui il corpus ITALIA NERA accoglie qui l'apparato. Nessuna interrogazione in rete effettuata. Vincolo fonti rispettato.</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>RICEZIONE E COLLOCAZIONE CERTIFICATA (21 documenti d'autore integrati in corpus/opera). Domini: D7 (Moro), D2/D3 (diaspora nazista, Sudafrica), D4 (P2/apparati).</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/ (21 file; nucleo: ALDO_MORO_APPENDICE_*_FASE_SETTIMA, PRIMA_SESSIONE_ESECUTIVA_TAVOLA_UNICA, Opera_Aldo_Moro_Tutta_la_Verita_Triangolazione)</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Raccordo Fase Settima (audit fonti Moro) con ITALIA NERA (voce 51)
Accertata l'identita' di metodo fra la Fase Settima del 'Registro dei
Cinquantacinque Giorni' e il corpus: i tre atti (produzione/acquisizione/
esposizione) e il collasso genealogico sono lo statuto Savona applicato
alle fonti. Crosswalk delle 10 appendici coi nodi del corpus (canale
orientale<->lodo Moro; falsificatore su 3 fascicoli<->Moro/Gladio/Ustica;
100 record servizio estero<->archivio CIA), e prova genealogica sulle
conclusioni balistiche (voci 35-39,48). DOCX + Excel di crosswalk.
Registro verifiche a voce 51.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2726,6 +2726,51 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>RACCORDO fra la FASE SETTIMA del 'Registro dei Cinquantacinque Giorni' (audit genealogico delle fonti del caso Moro) e ITALIA NERA - DOCX + Excel di crosswalk</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica (DOCX di raccordo) + repertorio (Excel di crosswalk)</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>IDENTITA' DI METODO accertata: i tre atti della Fase Settima (PRODUZIONE genera catena; ACQUISIZIONE = detenere non attestare; ESPOSIZIONE non accresce il computo) sono la formulazione piu' rigorosa dello statuto Savona; il COLLASSO GENEALOGICO (tre fonti di natura diversa NON sono tre catene indipendenti se risalgono al medesimo atto) e' la 'convergenza di milieu diverso da catena di comando' applicata alle FONTI. Regole letteralmente coincidenti: il non reperito non e' il distrutto/occultato (= reperto negativo voci 37,39); il rifiuto a comparire = constatazione negativa netta.</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>CROSSWALK delle 10 appendici possedute (seconda-dodicesima, manca prima e settima) con i nodi del corpus: app. ottava (canale orientale, quarta persona, Stato Zero di 4 apparati, XIII leg. doc. XXIII n.37) &lt;-&gt; lodo Moro/canale OLP (voce 40) e Hyperion; app. undicesima (falsificatore su 3 fascicoli: Moro, Ustica, struttura clandestina) &lt;-&gt; tre grandi nodi del corpus (balistica Moro voci 35-39/48; Gladio voci 41-42,44; Ustica); app. nona (100 record di un servizio estero, sala di lettura elettronica) &lt;-&gt; archivio cia.gov/readingroom in lista, distinzione indirizzo/atto. PROVA GENEALOGICA sulle conclusioni balistiche: confermate 'due armi' e 'PPK mai ritrovata'; il test spiega il declassamento gia' operato di 'Skorpion Dogali=arma di Moro' (voce 41, le molte esposizioni collassano su poche perizie); restano C il candidato di via Silvani (47/18) e il numero bossoli (indirizzo noto, atto non posseduto).</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: RACCORDO, non rifacimento; la Fase Settima non modifica i 70 Capitoli dell'opera Moro. Le due linee si scambiano profondita' (caso singolo) e ampiezza (trama). PENDENZE: mancano appendice PRIMA e SETTIMA (non caricate) - raccordo completo sulle 10 possedute, sospeso sulle 2 assenti; quarta persona non identificata e audizione 21.1.2000 non posseduta; 19 unita' non individuate (app. quarta) aperte = omologo archivistico della PPK mai ritrovata. Nessuna interrogazione in rete (ritorno al solo corpus, come prescrive la Tavola Unica). Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>RACCORDO CERTIFICATO (identita' di metodo fra le due linee; prova genealogica sulla balistica). Domini: D7, D2, D3, D4.</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica/ITALIA_NERA_RACCORDO_FASE_SETTIMA_MORO.docx + repertorio/ITALIA_NERA_RACCORDO_FASE_SETTIMA_MORO.xlsx</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ingresso appendice settima e aggiornamento raccordo Moro (voce 52)
Acquisita l'appendice settima alla Fase Settima (la Commissione dichiara
il proprio standard; XII legislatura, doc. XXIII n.1 e n.3, 1995) e sua
undicesima regola della risalita: 'la sede conferisce pubblicita', non
grado'. Fonda sulla dichiarazione della fonte la gradazione gia' adottata
dal corpus per gli atti delle Commissioni (A per acquisizioni, B per
ricostruzioni). Raccordo aggiornato (DOCX + Excel): completo su 11
appendici su 12, resta fuori la sola prima. Registro verifiche a voce 52.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2771,6 +2771,51 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>INGRESSO dell'APPENDICE SETTIMA (Fase Settima Moro) e AGGIORNAMENTO del raccordo con ITALIA NERA - resta fuori la sola appendice prima</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (appendice settima) + corpus/diagnostica + repertorio (raccordo aggiornato)</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Ricevuta e collocata in corpus/opera l'APPENDICE SETTIMA alla Fase Settima ('L'organismo successore e la dichiarazione del proprio standard'): opera sulle due relazioni semestrali della XII legislatura (doc. XXIII n.1 e n.3, 26.1 e 20.7.1995). CONTENUTO CARDINE: la Commissione DICHIARA il proprio standard - i suoi compiti non coincidono con quelli della magistratura, e puo' andare 'oltre la prova processuale', potenzialmente 'insufficiente o deformante' per fenomeni complessi. Da qui l'UNDICESIMA REGOLA DELLA RISALITA: quando un organo dichiara il proprio standard, il grado delle sue ricostruzioni si fissa su quella dichiarazione e non sull'autorevolezza della sede ('la sede conferisce pubblicita', non grado').</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>EFFETTO SUL CORPUS: la regola FONDA la gradazione gia' adottata (atti delle Commissioni = A per le acquisizioni documentali, B per ricostruzioni/valutazioni) sulla dichiarazione della FONTE medesima, non piu' sulla sola prudenza dell'autore - mutamento di natura, non di esito. Conferma la cautela della voce 40 (documenti parlamentari del filone Hyperion registrati ma proscioglimento -&gt; grado C). Il raccordo (DOCX + Excel di crosswalk) e' stato aggiornato: crosswalk esteso alla settima; nuovo paragrafo nel DOCX; pendenze corrette.</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: RACCORDO ora completo su UNDICI appendici su dodici; resta fuori la sola APPENDICE PRIMA (non caricata). La settima non modifica i 70 Capitoli (i settanta restano settanta). Restano non possedute la 'quarta persona' e l'audizione 21.1.2000; aperte le 19 unita' non individuate (app. quarta). Nessuna interrogazione in rete. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>INGRESSO E RACCORDO AGGIORNATI (11/12 appendici; undicesima regola della risalita fonda la gradazione del corpus). Domini: D7, D3, D4.</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/ALDO_MORO_APPENDICE_SETTIMA_FASE_SETTIMA.docx + raccordo aggiornato (DOCX + xlsx voce 51)</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ingresso appendici prima/14a/15a Fase Settima e aggiornamento raccordo (voce 53)
Acquisite tre nuove appendici Moro: la prima/base (Tavola accresciuta,
19 voci, Regola di Ferro = statuto Savona), la quattordicesima (schede
delle stragi 1969-1984, aggancio ai nodi-stragi della voce 45) e la
quindicesima (relazione XII leg. non discussa; corollario dell'undicesima
regola). Raccordo aggiornato (DOCX + Excel): completo su 14 appendici su
15, resta fuori la sola tredicesima. Registro verifiche a voce 53.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2816,6 +2816,51 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>INGRESSO di 3 nuove appendici della Fase Settima Moro (PRIMA/base, QUATTORDICESIMA, QUINDICESIMA) e AGGIORNAMENTO del raccordo - resta fuori la sola tredicesima</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (3 appendici) + corpus/diagnostica + repertorio (raccordo aggiornato)</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Ricevute e collocate (deduplicate; scartati numerosi doppioni di appendici gia' presenti): (1) APPENDICE PRIMA / base ('Appendice alla Fase Settima - Tavola accresciuta delle acquisizioni necessarie'): accresce il Capitolo 69 dell'opera Moro, iscrive le 19 voci con condizione di chiusura e di smentita, e formula la REGOLA DI FERRO ('dove la fonte documenta, l'opera certifica; dove la fonte tace, l'opera indaga e non afferma') = lo statuto Savona nella sua forma piu' nuda; (2) APPENDICE QUATTORDICESIMA ('La classe di comparazione che non c'e'): opera sulle schede informative delle STRAGI 1969-1984 (XI leg., 36 pagine), respingendo 'un errore che dispensa dal cercare'; (3) APPENDICE QUINDICESIMA ('La relazione che non fu discussa': terza relazione semestrale XII leg., doc. XXIII n.7, 21.2.1996): una proposta depositata e non discussa non acquista grado dal deposito.</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>AGGANCI AL CORPUS: la REGOLA DI FERRO (app. prima) e' identica allo statuto Savona (fondazione comune delle due linee); le STRAGI 1969-1984 (app. quattordicesima) sono i nodi-stragi gia' triangolati alla voce 45 (piazza Fontana, Bologna, piazza della Loggia, Peteano), e il rifiuto dell''errore che dispensa dal cercare' e' la non-inferenza del corpus; la quindicesima e' corollario dell'undicesima regola (la sede conferisce pubblicita', non grado). Raccordo (DOCX + Excel di crosswalk) aggiornato: crosswalk esteso a prima/quattordicesima/quindicesima; due nuovi paragrafi nel DOCX; pendenze corrette.</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: la serie Fase Settima si estende alla QUINDICESIMA; il corpus ne possiede ora QUATTORDICI (prima [base], seconda-dodicesima, quattordicesima, quindicesima). Resta fuori la sola appendice TREDICESIMA (non caricata): raccordo completo su 14, sospeso su 1. Le appendici non modificano i 70 Capitoli. Nessuna interrogazione in rete. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>INGRESSO E RACCORDO AGGIORNATI (14/15 appendici; Regola di Ferro = statuto Savona; stragi 1969-1984 agganciate alla voce 45). Domini: D7, D3, D4.</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/ALDO_MORO_APPENDICE_{PRIMA,QUATTORDICESIMA,QUINDICESIMA}_FASE_SETTIMA.docx + raccordo aggiornato (DOCX + xlsx)</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ingresso appendice tredicesima e chiusura della serie Fase Settima (voce 54)
Acquisita l'ultima appendice mancante (tredicesima, 'Una sola testimonianza
formale', Voce 46): dichiara e risolve per inferenza posizionale, verificata
su 5 ancoraggi, un difetto OCR degli ordinali delle sedute, correggendo la
dodicesima - modello da laboratorio della disciplina comune. Il corpus
possiede ora tutte le 15 appendici della Fase Settima: raccordo chiuso.
Registro verifiche a voce 54.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2861,6 +2861,51 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>INGRESSO dell'APPENDICE TREDICESIMA (Fase Settima Moro) e CHIUSURA della serie e del raccordo - il corpus possiede ora tutte le 15 appendici</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (appendice tredicesima) + corpus/diagnostica + repertorio (raccordo chiuso)</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Ricevuta e collocata l'APPENDICE TREDICESIMA ('Una sola testimonianza formale', Esecuzione della Voce quarantaseiesima): ricava dal prospetto analitico delle sedute l'oggetto delle 27 sedute i cui verbali non sono posseduti e individua fra gli auditi in sede formale le deposizioni che riguardano il caso. CASO METODOLOGICO LIMPIDO: DICHIARA un difetto della fonte (il riconoscimento ottico deforma gli indicatori ordinali - la prima seduta appare 18a, la seconda 24a, ecc.) e lo RISOLVE per inferenza posizionale, VERIFICATA su 5 ancoraggi indipendenti (processi verbali posseduti, es. 4a voce = 23.11.1988), dichiarando che 'la risoluzione e' un'inferenza dell'opera e non un dato del documento, ed e' falsificabile'; corregge l'appendice dodicesima in un punto che essa non sapeva spiegare.</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>AGGANCIO AL CORPUS: la vicenda e' un modello da laboratorio della disciplina comune - difetto della fonte dichiarato anziche' taciuto, errore plausibile riconosciuto come la specie peggiore, inferenza tenuta distinta dal dato, verifica su ancoraggi indipendenti, falsificabilita' offerta al lettore = la stessa operazione del corpus (registrare l'indirizzo e non il contenuto di un atto non posseduto; dichiarare falsificabile ogni ricostruzione). 'Una sola testimonianza formale' = conferma empirica del COLLASSO GENEALOGICO (poche deposizioni realmente sul caso fra i molti auditi). Raccordo (DOCX + Excel di crosswalk) aggiornato: crosswalk esteso alla tredicesima; due nuovi paragrafi nel DOCX; pendenze chiuse.</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: SERIE COMPLETA - il corpus possiede tutte le QUINDICI appendici della Fase Settima (prima/base, seconda-quindicesima); il raccordo e' CHIUSO, nessuna appendice manca. Restano aperte come pendenze INTERNE alle appendici (non del raccordo): la 'quarta persona' (app. ottava), l'audizione 21.1.2000 non posseduta, le 19 unita' non individuate (app. quarta) - code documentali dichiarate. Le appendici non modificano i 70 Capitoli. Nessuna interrogazione in rete. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>SERIE FASE SETTIMA COMPLETA (15/15) E RACCORDO CHIUSO. Domini: D7, D3, D4.</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/ALDO_MORO_APPENDICE_TREDICESIMA_FASE_SETTIMA.docx + raccordo chiuso (DOCX + xlsx)</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atto di ricezione: 12 documenti d'autore (registri Moro, dominiali, titanico) (voce 55)
Ingestione in corpus/opera di 12 file nuovi: la linea 'Registro Analitico
del caso Moro' in cinque versioni (V1/V3/V4/V5/V6) piu' il Registro
Speculare 'Anelli Profondi'; tre Registri Dominiali (D03 Intelligence,
D04 Massoneria, D08 Media); il Registro di Triangolazione Sacro-Guevara-
Moro; la Seconda Sequenza Giornaliera; e il generatore Node 'titanico'
dei 50 blocchi. Saltati i doppioni (raccordo Fase Settima, Tutta la
Verita' v2). Registro verifiche a voce 55.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2906,6 +2906,51 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>ATTO DI RICEZIONE: 12 documenti d'autore nuovi - la linea 'Registro Analitico del caso Moro' (V1/V3/V4/V5/V6 + Speculare), tre Registri Dominiali (D03/D04/D08), Sacro-Guevara-Moro, Seconda Sequenza Giornaliera, e il generatore 'titanico' dei 50 blocchi</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (ingesti con nome pulito)</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Ricevuti e collocati in corpus/opera 12 file nuovi (saltati per contenuto identico i 2 ri-caricamenti del mio raccordo Fase Settima e la Tutta la Verita' v2). LINEA REGISTRO ANALITICO DEL CASO MORO ('Registro autonomo delle reti informali del sequestro e dell'omicidio di Aldo Moro'), versioni progressive: V1 Integrale, V3 con secondo anello, V4 'salto della quaglia', V5 'rinnovamento cartesiano', V6 'apporto kuhniano' (manca V2, non caricata), piu' REGISTRO SPECULARE 'Anelli Profondi' V1 (dal secondo al quarto anello di prossimita'). TRE REGISTRI DOMINIALI 'delle Reti Informali Transnazionali': D03 Intelligence, D04 Massoneria, D08 Media (2 ago 2026). ITALIA_NERA_REGISTRO_DI_TRIANGOLAZIONE_SACRO_GUEVARA_MORO (23 ago; 'Il Sacro, il Dossier Guevara e i Dossier Moro'). ITALIA_NERA_OPERA_SECONDA_SEQUENZA_GIORNALIERA_PARTE_PRIMA ('Tutta la Verita' - prosecuzione titanica').</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>GENERATORE: OPERA_ALDO_MORO_TUTTA_LA_VERITA_TITANICO_50_BLOCCHI_generatore.js - script Node/docx d'autore (De Michele) che genera 'Approfondimento titanico della triangolazione in cinquanta blocchi mirati' (10 parti, 50 blocchi), condotto sui tre reperti (Opera del 22 ago; Dossier V74 del 19 ago, 17a tavola; Trattato Topografico), con impronte SHA-256 dichiarate e la REGOLA DI FERRO in ogni blocco. E' la sorgente di un documento dell'opera: conservato con la linea Moro.</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: ATTO DI RICEZIONE, non verifica; conservazione cumulativa (nulla si cancella). Le versioni progressive del Registro Analitico si conservano tutte (manca V2). I tre Registri Dominiali (D03/D04/D08) arricchiscono i domini del corpus e potranno alimentare un aggiornamento del registro analitico integrale dei nodi (voce 47). Nessuna interrogazione in rete. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>RICEZIONE E COLLOCAZIONE CERTIFICATA (12 documenti d'autore + 1 generatore in corpus/opera). Domini: D7 (Moro), D3 (Intelligence), D4 (Massoneria), D8 (Media).</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/ (REGISTRO_ANALITICO_CASO_MORO_V1..V6 + SPECULARE; REGISTRO_DOMINIALE_D03/D04/D08; SACRO_GUEVARA_MORO; SECONDA_SEQUENZA_GIORNALIERA; titanico generatore)</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atto di ricezione maggiore: 556 schede-nodo + Registro Sinaptico Generale (voce 56)
Ingestione di 556 dossier per-nodo (DOCUMENTO-NODO del Registro Integrale
V63, con dominio e grado Savona), estratti da 10 ZIP e ordinati in
corpus/opera/nodi/<dominio> (D02 305, D03 58 + sinaptico 58, D09 44,
D06 23, D10 22, D05 16, D04 10 + sinaptico 10, D08 7, D01/D02 singole),
piu' il Registro Sinaptico Generale (il connettoma dell'opera, 78k
parole). E' la base granulare che espande il registro analitico
integrale dei nodi (voce 47). Registro verifiche a voce 56.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2951,6 +2951,51 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>ATTO DI RICEZIONE MAGGIORE: 556 schede-nodo per dominio (DOCUMENTO-NODO del Registro Integrale V63) + il REGISTRO SINAPTICO GENERALE ('il connettoma dell'opera')</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/nodi/&lt;dominio&gt; (schede) + corpus/opera (registro sinaptico generale)</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Ricevuti e collocati 556 dossier per-nodo (ciascuno 'DOCUMENTO-NODO' del Registro Integrale V63, con dominio primario e grado Savona conservato dalla sede d'origine), estratti da 10 archivi ZIP e ordinati in corpus/opera/nodi/&lt;dominio&gt;: D02 (attori geopolitici e regimi) 305 schede; D03 (intelligence e servizi) 58 + D03 SINAPTICO 58; D09 (assi militari) 44; D06 (reti bancarie/finanza) 23; D10 (magistratura/giustizia) 22; D05 (religione/matrici) 16; D04 (massoneria) 10 + D04 SINAPTICO 10; D08 (media) 7; D01 (criminalita' organizzata: Riina) 1 + SINAPTICO 1; D02 SINAPTICO (Andreotti) 1. Deduplicato un ZIP D08 identico (stesso md5). Aggiunte le schede singole Riina (D01) e Andreotti (D02) con le loro varianti sinaptiche.</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>REGISTRO SINAPTICO GENERALE (78.231 parole): 'il connettoma dell'opera' - elenco integrale delle sinapsi per co-occorrenza rilevate dalla cascata sui tredici registri della Conoscenza di Progetto, con la matrice delle coppie di dominio e la gerarchia dei nodi per grado sinaptico. E' la versione d'autore, granulare e completa, del concetto di nodo/sinapsi che il corpus aveva consolidato nel registro analitico integrale (voce 47, 260 nodi): questa collezione lo espande a oltre 550 schede monografiche piu' il connettoma generale.</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: ATTO DI RICEZIONE, non verifica; conservazione cumulativa. I gradi Savona delle schede sono attribuiti nella sede d'origine (Registro Integrale V63) e qui conservati senza eccezioni. FOLLOW-UP possibile: federare queste schede e il connettoma con il registro analitico integrale dei nodi (voce 47), aggiornandolo dalla base granulare V63. Nessuna interrogazione in rete. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>RICEZIONE MAGGIORE CERTIFICATA (556 schede-nodo + connettoma generale in corpus/opera). Domini: tutti (D01-D10).</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/nodi/ (556 DOCUMENTO-NODO in 13 cartelle di dominio) + corpus/opera/ITALIA_NERA_REGISTRO_SINAPTICO_GENERALE_2AGO2026.docx</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atto di ricezione: 15 documenti d'autore (opera-madre Moro, registri, PDF V63) (voce 57)
Ingestione in corpus/opera di 15 file: l'opera-madre 'Aldo Moro - Tutta
la verita / Una guerra senza fine' (374.593 parole); il Registro Analitico
Caso Moro V11 e lo Speculare V4; quattro registri di metodo (Analitico
Rete, Vaglio Fascia Prima, Pattern Avanzati, Neuroni Neonati); tre
triangolazioni (Tre Famiglie, Corpus, Registro Esteso); 'Il Sacro e
l'Eversione'; 'Maestri Cosmici'; 'Canale Petrolifero' (Chiavelli/Lucina);
e due PDF di verifica della base V63. Registro verifiche a voce 57.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2996,6 +2996,51 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>ATTO DI RICEZIONE: 15 documenti d'autore (l'opera-madre 'Aldo Moro - Tutta la verita' / Una guerra senza fine' da 374.593 parole; Registro Analitico Caso Moro V11 e Speculare V4; registri di metodo; triangolazioni; 'Il Sacro e l'Eversione'; 'Canale Petrolifero'; due PDF V63)</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (ingesti con nome pulito; PDF inclusi)</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Ricevuti e collocati 15 file nuovi (deduplicato un doppione interno: REGISTRO_TRIANGOLAZIONE_CORPUS 1=2). OPERA-MADRE: 'Aldo_Moro_Tutta_la_verita - Una guerra senza fine' (374.593 parole) - il grande testo integrale del caso Moro. LINEA REGISTRO ANALITICO CASO MORO: V11 'Applicazione definitiva' (38.467 parole, ultima versione) e Speculare V4 'Applicazione definitiva' (Anelli Profondi, edizione seconda). REGISTRI DI METODO: Registro Analitico Rete; Registro di Vaglio (Fascia Prima); Registro dei Pattern Avanzati; Registro dei Neuroni Neonati. TRIANGOLAZIONI: Tre Famiglie in cinquanta blocchi; Registro di Triangolazione del Corpus ('Spine, ambienti e Stati Zero'); Opera Aldo Moro - Registro Esteso di Triangolazione. TEMATICI: 'Il Sacro e l'Eversione' (esoterismo/religione/metafisica nella storia nera, D10); 'Dossier Maestri Cosmici - Aetherius Society, dieci testimonianze'; 'Canale Petrolifero in dieci capitoli' (nodo Chiavelli, contratto Lucina, intermediari privati - area ENI/energia, D6).</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>DUE PDF: 'ITALIA_NERA_Registro_Verifica_Triangolazione_V63' (512 KB) e 'ITALIA_NERA_REGISTRO_TRIANGOLAZIONE_CONFERIMENTO_23AGO2026' (130 KB) - registri di verifica/conferimento della base V63, collocati in corpus/opera accanto alle schede-nodo V63 (voce 56). Tutti i documenti si ancorano al 'Registro Integrale V63' e alla Regola di Ferro.</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: ATTO DI RICEZIONE, non verifica; conservazione cumulativa (nulla si cancella; le versioni Moro V1-V6 e V11 coesistono). FOLLOW-UP: 'Il Sacro e l'Eversione' e 'Maestri Cosmici' arricchiscono il dominio D10 (matrici dottrinali/esoteriche); 'Canale Petrolifero' (Chiavelli/Lucina) e' un nodo D6 (energia/finanza) triangolabile con la dorsale gas-energia (voci 44-46). Nessuna interrogazione in rete. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>RICEZIONE CERTIFICATA (13 DOCX + 2 PDF in corpus/opera; opera-madre Moro inclusa). Domini: D7 (Moro), D10 (sacro/esoterismo), D6 (petrolifero), D1-D3 (triangolazioni).</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/ (Aldo_Moro_Tutta_la_verita_Una_guerra_senza_fine; REGISTRO_ANALITICO_CASO_MORO_V11; REGISTRO_SPECULARE_V4; registri di metodo e triangolazione; IL_SACRO_E_L_EVERSIONE; CANALE_PETROLIFERO; 2 PDF V63)</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Triangolazione totale: connettoma V63 vs classifica per frequenza (voce 58)
Confronto fra due metodi indipendenti: la classifica per frequenza
(voce 46) e il connettoma d'autore V63 per grado sinaptico. Convergenza
certificata sul nucleo di hub dello Stato profondo italiano (Gelli,
Moro, Delle Chiaie, Andreotti, Pinochet, Ordine Nuovo); divergenza
spiegata (lobo internazionale vs lobo istituzionale = struttura
bicefala). Sinapsi inter-dominio maestre = i ponti del corpus misurati
(SID-ON, Gelli-Sindona-IOR-Ambrosiano, Andreotti-Falcone). Riconcilia-
zione del dominio D10 (magistratura). Statuto Savona anche sul
connettoma (PCC-PCC = omonimia). DOCX + Excel. Registro a voce 58.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3041,6 +3041,51 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE TOTALE: il connettoma d'autore V63 (grado sinaptico) e le triangolazioni del corpus (frequenza, voce 46) a confronto - DOCX + Excel</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica (DOCX) + repertorio (Excel a 6 fogli)</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>DUE METODI INDIPENDENTI a confronto: (a) la mia classifica per FREQUENZA di menzione (voce 46), (b) il CONNETTOMA V63 per GRADO SINAPTICO (numero di neuroni distinti connessi sui 13 registri). Gerarchia V63: CIA (159), Gelli (152), Moro (151), Andreotti (146), Lucky Luciano (143), Trump (129), Delle Chiaie (122), Falcone (118), Sindona (113), Banco Ambrosiano (113), SISMI (111), Ordine Nuovo (109), SID (105), Salvo Lima (103), Di Bernardo, Maletti, Riina, Gioia, Magliana, Pinochet. CONVERGENZA CERTIFICATA: entrambi i metodi collocano ai vertici Gelli, Moro, Delle Chiaie, Andreotti, Pinochet, Ordine Nuovo (nucleo di hub dello Stato profondo italiano). DIVERGENZA SPIEGATA: la mia frequenza illumina il lobo INTERNAZIONALE (Aginter/apartheid/euroasia), il connettoma il lobo ISTITUZIONALE ITALIANO (Stato-mafia-P2-Vaticano). Struttura BICEFALA confermata da due metodi.</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>SINAPSI INTER-DOMINIO MAESTRE = i ponti del corpus, misurati: SID-Ordine Nuovo (141) = porosita' Stato-eversione (cerniera Giannettini, voci 45,48); quadrilatero Gelli-Sindona-IOR-Banco Ambrosiano (101-135) = cluster P2-Vaticano-finanza (in parte da triangolare); Andreotti-Falcone (119) = politica-magistratura; SCU-Corona (176) = mafia-massoneria. Trump 6o nel connettoma = aggancio alla dorsale euroasiatica (voci 45-46). INNESTI TEMATICI NUOVI: 'Il Sacro e l'Eversione' e 'Maestri Cosmici' (esoterismo, aggancio alla matrice religiosa di Aginter, Fase I); 'Canale Petrolifero' (Chiavelli/Lucina, energia D6, triangolabile con dorsale gas ed con Sindona/Ambrosiano).</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>RICONCILIAZIONE TASSONOMICA: la base V63 e' autoritativa; coincide col registro voce 47 tranne il DOMINIO D10, che in V63 e' MAGISTRATURA (Falcone, Caponnetto, Terranova) e non 'matrici dottrinali' - il registro voce 47 va riallineato. STATUTO SAVONA ANCHE SUL CONNETTOMA: la sinapsi piu' intensa (PCC-PCC, 193) e' un REPERTO DI OMONIMIA (sigla, non nesso), non un ponte storico - nessuna misura dispensa dal giudizio. VERDETTO-CARDINE INVARIATO: convergenza di milieu/sistema certificata (ora da 2 metodi); catena di comando unica NON provata; arco negativo galassia nera&lt;-&gt;Putin permane (solo ponte euroasiatico). Nessuna interrogazione in rete. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE TOTALE CERTIFICATA (2 metodi indipendenti convergenti; struttura bicefala; riconciliazione domini). Domini: tutti (D1-D10).</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica/ITALIA_NERA_TRIANGOLAZIONE_TOTALE_V63.docx + repertorio/ITALIA_NERA_TRIANGOLAZIONE_TOTALE_V63.xlsx</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atto di ricezione: documenti fondativi V63 (registro-madre 1,4M parole) (voce 59)
Ingestione dei sei documenti fondativi della base V63: il Registro
Integrale V63 (registro-madre dei nodi, 1.417.722 parole, sorgente
autoritativa delle 556 schede e del connettoma), il V67 Tomo 1 Titanico
(193k parole), la Nota Metodologica (premessa epistemologica), la scheda
diagnostica, e due triangolazioni (Seconda Serie Ricognizioni, Schede-
Dossier). Completa l'architettura V63 e abilita il riallineamento del
registro voce 47. Registro verifiche a voce 59.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3086,6 +3086,51 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>ATTO DI RICEZIONE: i documenti FONDATIVI della base V63 - il REGISTRO INTEGRALE V63 (registro-madre, 1.417.722 parole), il V67 Tomo 1 Titanico, la Nota Metodologica, e tre triangolazioni V63</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (ingesti con nome pulito)</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Ricevuti e collocati 6 file fondativi (deduplicato un doppione: Seconda Serie Ricognizioni caricata due volte). PEZZO CARDINE: ITALIA_NERA_REGISTRO_INTEGRALE_V63 (1.417.722 parole, 3,6 MB) - il registro-madre dei nodi da cui derivano le 556 schede della voce 56 e il connettoma della voce 56; e' la SORGENTE AUTORITATIVA dell'intera base V63. ITALIA_NERA_V67_TOMO_1_TITANICO_V63 (193.384 parole, 'Edizione Integrale Federata', Tomo 1). ITALIA_NERA_V63_NOTA_METODOLOGICA_E_SEZIONI (19.440 parole: premessa epistemologica, il problema della conoscenza nel caso Moro, e la partizione in sezioni). ITALIA_NERA_V63_SCHEDA_DIAGNOSTICA_PMI (scheda diagnostica complessiva). TRIANGOLAZIONE SECONDA SERIE - Ricognizioni ('le diciotto ricognizioni'). TRIANGOLAZIONE SCHEDE-DOSSIER V63 ('la sesta tavola').</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETAMENTO DELLA BASE V63: con questi documenti il corpus possiede ora l'intera architettura V63 - il registro-madre (voce 59), le 556 schede-nodo e il connettoma (voce 56), i registri di metodo e verifica (voci 57-59), le triangolazioni d'autore. La Nota Metodologica fornisce la premessa epistemologica esplicita che fonda tutto l'impianto. Questi documenti ABILITANO DEFINITIVAMENTE il riallineamento del registro analitico integrale dei nodi (voce 47) alla tassonomia autoritativa V63 (compreso il D10 = Magistratura, gia' rilevato alla voce 58).</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: ATTO DI RICEZIONE, non verifica; conservazione cumulativa. Il REGISTRO INTEGRALE V63 e' la sorgente autoritativa: ogni futura verifica o federazione dei nodi attinge ad esso. Nessuna interrogazione in rete. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>RICEZIONE CERTIFICATA (6 documenti fondativi V63, compreso il registro-madre da 1,4 milioni di parole). Domini: tutti (D1-D10).</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/ (REGISTRO_INTEGRALE_V63; V67_TOMO_1_TITANICO_V63; V63_NOTA_METODOLOGICA_E_SEZIONI; V63_SCHEDA_DIAGNOSTICA_PMI; TRIANGOLAZIONE_SECONDA_SERIE_RICOGNIZIONI_V63; TRIANGOLAZIONE_SCHEDE_DOSSIER_V63)</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Registro Unico dei Nodi: federazione base V63 e sintesi corpus (voce 60)
Federati in un unico registro autoritativo 753 nodi: le 486 schede-nodo
di base V63, i nodi della sintesi (voce 47) non coperti, e i 40 hub del
connettoma con grado sinaptico. Tassonomia V63 autoritativa con D10
riconciliato a Magistratura (Falcone, Borsellino). Lacuna dichiarata:
schede D7 non caricate (nodi da voce 47/connettoma). Strumento di ordine,
non di accertamento. DOCX + Excel a 4 fogli. Registro verifiche a voce 60.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3131,6 +3131,51 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>REGISTRO UNICO DEI NODI: federazione della base V63 (486 schede + connettoma) e della sintesi del corpus (voce 47) in un solo registro autoritativo - DOCX + Excel</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica (DOCX) + repertorio (Excel del registro unico)</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>753 NODI federati in un unico registro, ordinati per dominio e per grado sinaptico. FONTI dichiarate per ciascun nodo: 486 schede-nodo di base del Registro Integrale V63 (voci 56,59), i nodi della sintesi del corpus (registro voce 47) non gia' coperti, e i 40 nodi di grado sinaptico massimo annotati dal connettoma. Distribuzione (tassonomia V63): D1=70, D2=351, D3=85, D4=27, D5=16, D6=56, D7=49, D8=11, D9=56, D10=32. RICONCILIAZIONE DEFINITIVA: la base V63 e' autoritativa; il D10 e' MAGISTRATURA E GIUSTIZIA (Falcone, Borsellino, Caponnetto, Terranova, Saetta, Caccia), non 'matrici dottrinali'; la religione e' D5 (con lo IOR); le matrici dottrinali restano materia tematica.</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>LACUNA DICHIARATA: le schede del dominio D7 (eversione nera) NON sono state caricate nella base V63; i suoi 49 nodi provengono qui dalla sintesi voce 47 e dal connettoma (Delle Chiaie, Ordine Nuovo, BR, AN, Vinciguerra - tutti alti per grado sinaptico) - da completare con le schede V63 del D7 quando disponibili. Il registro unico rende visibile la struttura bicefala: i 40 hub di grado massimo sono in larga parte l'intreccio istituzionale italiano (CIA, Gelli, Moro, Andreotti, Sindona, Ambrosiano, servizi, magistratura), con i nodi dell'eversione nera come cerniera verso il lobo internazionale e il nodo Trump come cerniera verso la dorsale euroasiatica.</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: strumento di ORDINE, non di accertamento; registra nodi/fonti/domini/centralita', non promuove gradi ne' trasforma centralita' in colpa. Il grado sinaptico e' misura di connessione, distinto dal grado probatorio Savona (le schede V63 recano quasi tutte A dalla sede d'origine). Regola di Ferro comune alle due opere. Il registro unico sussume le due anagrafi (voce 47 e base V63) senza cancellarle (restano fonti). Nessuna interrogazione in rete. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>REGISTRO UNICO DEI NODI GENERATO E CERTIFICATO (753 nodi, 10 domini, 40 hub, tassonomia V63 riconciliata). Domini: tutti (D1-D10).</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica/ITALIA_NERA_REGISTRO_UNICO_NODI_V63.docx + repertorio/ITALIA_NERA_REGISTRO_UNICO_NODI_V63.xlsx</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atto di ricezione: Terza Serie Moro e Tomi 2-4 del V67 Titanico V63 (voce 61)
Ingestione di 4 file nuovi (gli altri del lotto erano ri-caricamenti):
la Terza Serie di triangolazione sul caso Moro e i Tomi 2 (472k parole),
3 (141k) e 4 (614k) dell'edizione integrale federata V67 Titanico V63.
Con il Tomo 1 gia' in repo, l'edizione titanica in quattro tomi (~1,42M
parole) e' ora completa - forma editoriale del registro-madre V63.
Registro verifiche a voce 61.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3176,6 +3176,51 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>ATTO DI RICEZIONE: la Terza Serie di triangolazione sul caso Moro e i Tomi 2, 3, 4 del V67 Titanico V63 (edizione integrale federata) - completano l'edizione titanica in quattro tomi</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (ingesti con nome pulito)</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Ricevuti e collocati 4 file nuovi (tutti gli altri del lotto erano ri-caricamenti gia' in repo, compreso il mio Registro Unico dei Nodi, la Nota Metodologica, il Tomo 1, la Seconda Serie e la Schede-Dossier). ITALIA_NERA_TRIANGOLAZIONE_TERZA_SERIE_CASO_MORO_V63 (3.192 parole): la terza serie di triangolazione dedicata al caso Moro. I TRE TOMI mancanti dell'EDIZIONE INTEGRALE FEDERATA 'V67 Titanico V63': Tomo 2 (472.029 parole), Tomo 3 (140.820 parole), Tomo 4 (614.240 parole). Con il Tomo 1 (193.384 parole, gia' in repo alla voce 59) l'edizione titanica in quattro tomi e' ora COMPLETA nel corpus, per un totale di circa 1,42 milioni di parole - la versione federata e impaginata del Registro Integrale V63 (voce 59).</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETAMENTO DELL'EDIZIONE V67 TITANICO: i quattro tomi sono la forma editoriale definitiva della base V63 (il registro-madre da 1,4 milioni di parole della voce 59, qui articolato in quattro volumi). Con questo ingresso il corpus possiede l'intera base V63 sia in forma di registro-madre unico, sia in forma di edizione federata in quattro tomi, sia in forma di 556 schede-nodo e connettoma (voce 56), sia nel Registro Unico dei Nodi che le federa (voce 60).</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: ATTO DI RICEZIONE, non verifica; conservazione cumulativa. La Terza Serie sul caso Moro si aggiunge alla Prima e alla Seconda (Ricognizioni) gia' in corpus. Nessuna interrogazione in rete. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>RICEZIONE CERTIFICATA (Terza Serie Moro + Tomi 2-4 del V67 Titanico; edizione in 4 tomi completa). Domini: tutti (D1-D10), D7 (Moro).</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/ (TRIANGOLAZIONE_TERZA_SERIE_CASO_MORO_V63; V67_TOMO_2/3/4_TITANICO_V63)</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atto di ricezione: dittico P2 V61 (elenco verificato + analisi di non-uso) (voce 62)
Ingestione di due documenti V61: l'Elenco P2 verificato (960/962 record
dalla fonte reale Anselmi/Castiglion Fibocchi, grado A, corregge tre
attribuzioni del Registro V61) in corpus/opera; e l'Analisi Strutturale
che motiva il non-uso di due liste massoniche anonime (reperto negativo:
non verificabilita') in corpus/diagnostica. Dittico esemplare dello
statuto Savona - fonte verificabile usata, liste anonime respinte;
nessun nominativo di massa entra nel corpus. Registro verifiche a voce 62.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3221,6 +3221,51 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>ATTO DI RICEZIONE di un dittico metodologico V61: l'ELENCO P2 verificato (fonte Anselmi/Castiglion Fibocchi, grado A) e l'ANALISI STRUTTURALE che motiva il NON-USO di due liste massoniche anonime (reperto negativo)</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (elenco P2) + corpus/diagnostica (analisi strutturale)</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>ELENCO_P2_FASCICOLI_VERIFICATO_V61 (corpus/opera, D4): estrazione dalla FONTE REALE - 960 record su 962, ordinati per numero di fascicolo, dall'elenco alfabetico sequestrato a Castiglion Fibocchi il 17.3.1981 e pubblicato in allegato alla Relazione della Commissione parlamentare d'inchiesta presieduta da Tina Anselmi (comunicata alle Camere il 12.7.1984). GRADO A (fonte verificabile). Corregge tre attribuzioni del Registro V61 e risponde empiricamente alla domanda sull'adiacenza numerica dei fascicoli.</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>ANALISI_STRUTTURALE_FILE_CARICATI_V61 (corpus/diagnostica): diagnosi di provenienza, portata e qualita' di due PDF di elenchi massonici (308 e 2.206 pagine) condotta SENZA estrarre alcun nominativo, che documenta e motiva la DECISIONE DI NON UTILIZZARLI COME FONTE - privi di intestazione, data, riferimento a operazione giudiziaria o qualunque marcatura di riconducibilita' a fonte verificabile; e sono due esportazioni del medesimo archivio (non due fonti indipendenti). E' un REPERTO NEGATIVO dichiarato (non verificabilita' + riservatezza): il corpus registra la decisione di non-uso come risultato.</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: DITTICO ESEMPLARE dello statuto Savona - una fonte verificabile (Anselmi/Castiglion Fibocchi) e' USATA e graduata A; due liste anonime sono RESPINTE con motivazione dichiarata. NB: NESSUN nominativo di massa entra nel corpus - le liste massoniche anonime NON sono ingerite, solo l'analisi d'autore che ne motiva l'esclusione. Il P2 verificato alimenta il dominio D4 (massoneria) e corregge il Registro V61. Nessuna interrogazione in rete. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>RICEZIONE CERTIFICATA (dittico P2: elenco verificato grado A + analisi con decisione di non-uso dichiarata). Domini: D4 (massoneria/P2).</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/ITALIA_NERA_ELENCO_P2_FASCICOLI_VERIFICATO_V61.docx + corpus/diagnostica/ITALIA_NERA_ANALISI_STRUTTURALE_FILE_CARICATI_V61.docx</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atto di ricezione: Registro Dominiale D07 Terrorismo (voce 63)
Ingestione del Registro Dominiale del Dominio 7 (terrorismo e violenza
politica, partizione V63, 6.827 parole): l'omologo D7 dei registri
dominiali D3/D4/D8. Colma parzialmente la lacuna D7 dichiarata alla voce
60 - il dominio eversione nera/rossa entra ora in forma di registro di
dominio; restano da acquisire le schede-nodo singole del D7 (ZIP non
caricabile). Registro verifiche a voce 63.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3266,6 +3266,51 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>ATTO DI RICEZIONE: il REGISTRO DOMINIALE D07 - Terrorismo e violenza politica (partizione V63) - colma PARZIALMENTE la lacuna del dominio D7 dichiarata alla voce 60</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (registro dominiale)</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Ricevuto e collocato (deduplicato: caricato due volte, identico) il REGISTRO DOMINIALE DEL DOMINIO 7 - TERRORISMO E VIOLENZA POLITICA (6.827 parole), 'area cerebrale D7 della struttura neuronale dell'opera', partizione del Registro Integrale V63. Documenta l'area D7 con i suoi nodi (eversione nera e rossa: Delle Chiaie, Ordine Nuovo, Brigate Rosse, Avanguardia Nazionale, Vinciguerra...), gli archi cross-section e la cronologia marcata. E' l'omologo D7 dei registri dominiali D03/D04/D08 gia' ricevuti (voce 55).</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>EFFETTO SULLA LACUNA D7: alla voce 60 (Registro Unico dei Nodi) il dominio D7 era presente solo 'di seconda mano' (dalla sintesi voce 47 e dal connettoma), perche' le schede-nodo singole del D7 non erano state caricate. Questo registro dominiale porta ora il D7 nel corpus in FORMA DI REGISTRO DI DOMINIO (non ancora come schede singole): la lacuna e' COLMATA PARZIALMENTE. RESTA DA ACQUISIRE: le schede-nodo individuali del D7 (l'archivio ZIP non si carica - da ritentare o da committare direttamente nel repo).</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: ATTO DI RICEZIONE, non verifica; conservazione cumulativa. Il registro dominiale D7 e' fonte autoritativa V63 per l'area terrorismo, coerente con i domini gia' ricevuti. Con questo il corpus possiede i registri dominiali per D3, D4, D7, D8 (mancano ancora D1, D2, D5, D6, D9, D10 come registri dominiali autonomi, benche' le loro schede siano gia' in corpus). Nessuna interrogazione in rete. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>RICEZIONE CERTIFICATA (registro dominiale D7; lacuna D7 colmata a livello di dominio, schede singole ancora attese). Domini: D7 (eversione/terrorismo).</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/ITALIA_NERA_REGISTRO_DOMINIALE_D07_TERRORISMO_2AGO2026.docx</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Triangolazione cluster P2-Vaticano-finanza (Gelli-Sindona-Calvi-IOR) (voce 64)
Sviluppato il grande nodo italiano finora solo annunciato: il quadrilatero
Gelli/P2 - Sindona - Calvi/Ambrosiano - IOR/Marcinkus, dalle schede V63
grado A. Spina = Arco #10 certificato (Sindona-Calvi->IOR->estero);
scia di sangue (Ambrosoli 1979, Calvi 1982, Sindona 1986); conferma dal
connettoma (Gelli-Sindona 135, IOR-Sindona 134, CIA-IOR 129...);
triangolazione verso mafia D1, Condor, atlantico, magistratura D10,
stragi (Gelli mandante Bologna). DOCX + Excel. Registro a voce 64.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3311,6 +3311,51 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE del cluster P2-VATICANO-FINANZA (Gelli/P2 - Sindona - Calvi/Ambrosiano - IOR/Marcinkus) - il grande nodo italiano finora annunciato e non sviluppato - DOCX + Excel</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica (DOCX) + repertorio (Excel a 6 fogli)</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>QUADRILATERO a 4 vertici, dalle schede V63 grado A: Licio Gelli (D4, Venerabile P2, lista Castiglion Fibocchi 17.3.1981, 962 affiliati, pregresso fascista/CIA/Argentina); Michele Sindona (D6, banchiere P2, Banca Privata Italiana + Franklin National Bank/David Kennedy, ergastolo per Ambrosoli, avvelenato in carcere 22.3.1986); Roberto Calvi (D6, Banco Ambrosiano, P2, impiccato a Blackfriars 18.6.1982, sentenza 2007 = omicidio mandato Calo'); IOR/Marcinkus (D5, banca vaticana, presidenza 1971-1989, FBI legami Chicago Outfit, lettere di patronato a off-shore Calvi 1981, immunita' lateranense). SPINA = ARCO #10 GIA' CERTIFICATO A: Sindona-Calvi -&gt; IOR -&gt; banchi vaticani -&gt; estero (Filiazione). SCIA DI SANGUE: Ambrosoli 1979 (mandato Sindona), Calvi 1982 (mandato Calo'), Sindona 1986 (avvelenato).</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>CONFERMA DAL CONNETTOMA (sinapsi piu' intense): Gelli-Sindona 135, IOR-Sindona 134, CIA-IOR 129, IOR-Ambrosiano 121, Andreotti-Gelli 116, Gelli-IOR 101. TRIANGOLAZIONE COL CORPUS: verso D1 mafia (Sindona riciclatore, Calvi/Calo', Marcinkus/Chicago) = ponte finanza-criminalita'; verso Condor/galassia nera (Gelli fascista, P2 in Argentina/Massera-Suarez Mason, voce 40); verso l'atlantico (CIA, Franklin/Kennedy); verso D10 magistratura (Ambrosoli caso simbolo dell'omicidio del servitore che documenta, come Falcone/Borsellino); verso le stragi (Gelli mandante di Bologna, voce 48).</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: triangolazione condotta sul SOLO CORPUS (schede V63 grado A + connettoma), senza interrogazione in rete. CERTO (A): identita'/legami, Arco #10, omicidio Ambrosoli+ergastolo Sindona, omicidio Calvi (sentenza 2007), avvelenamento Sindona, crack Ambrosiano, lettere IOR-Calvi, Gelli mandante Bologna. RESTA B/C: mandante ultimo oltre l'esecutore, responsabilita' penale IOR/Marcinkus (immunita' lateranense, mai processati in Italia), nesso Andreotti-cluster (Livello C, appaiamento automatico), regia complessiva. Convergenza di milieu certificata; catena di comando unica non provata. Cifra: e' il VOLTO FINANZIARIO dello Stato profondo (l'arma e' il denaro, il metodo il riciclaggio, la scia di sangue e la protezione istituzionale le stesse degli altri fronti). Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE CERTIFICATA (cluster P2-Vaticano-finanza; quadrilatero, arco-spina, scia di sangue, conferma connettoma). Domini: D4, D5, D6, D1, D2, D10.</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica/ITALIA_NERA_TRIANGOLAZIONE_P2_VATICANO_FINANZA.docx + repertorio/ITALIA_NERA_TRIANGOLAZIONE_P2_VATICANO_FINANZA.xlsx</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atto di ricezione: 4 fonti primarie in fonti/ con gradazione differenziata (voce 65)
Ingestione di 4 fonti primarie: l'atto parlamentare 'Memoria Condivisa'
(De Luca, Commissione stragi XIII leg., Doc XXIII n.64; A acquisizione/
B valutazione), il saggio accademico Cross 2016 sul caso Cirillo e la
Camorra (B), l'articolo di la Repubblica sui mandanti del 2 agosto
(B/C) e il 'Memoriale di un Gladiatore' da blog (C con riserva di
attendibilita'). Gradazione differenziata dichiarata. Registro a voce 65.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3356,6 +3356,51 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>ATTO DI RICEZIONE di 4 FONTI PRIMARIE in fonti/ (atto parlamentare 'Memoria Condivisa', saggio accademico sul caso Cirillo, articolo di stampa sul 2 agosto, memoriale Gladio da blog) - con gradazione differenziata</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>fonti/ (atti e fonti acquisiti da terzi)</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Ricevute e collocate in fonti/ 4 fonti primarie uniche (deduplicata la Memoria Condivisa, caricata 4 volte): (1) XIII_leg_Doc_XXIII_64_Vol_I_Tomo_IV_p375_Memoria_Condivisa (9.351 parole): ATTO PARLAMENTARE - Commissione stragi XIII legislatura, Doc. XXIII n.64, Vol I Tomo IV pp.375-408, 'Il problema di definire una memoria storica condivisa', elaborato del senatore Athos De Luca. GRADO: A per l'acquisizione (atto pubblicato), B per le valutazioni (elaborato = ricostruzione, per l'undicesima regola della risalita). (2) Storiaememoria.pdf (50 pagine): SAGGIO ACCADEMICO - rivista Cross Vol.2 N.3 (2016), DOI 10.13130/cross-7795, 'La Camorra e il caso Cirillo' a cura di Sarah Mazzenzana, con estratti dal Rapporto parlamentare sulla Camorra. GRADO B (accademico, peer-reviewed). Aggancio: il caso Cirillo (sequestro BR 1981, mediazione Cutolo/Camorra-DC-servizi) - nodo che lega BR, Camorra (D1), DC (D2) e servizi (D3).</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>(3) Due_agosto_a_un_passo_dai_mandanti_la_Repubblica.mht: ARTICOLO DI STAMPA (bologna.repubblica.it, 2.8.2013) sui mandanti della strage di Bologna. GRADO B/C (fonte giornalistica; la Repubblica NON e' fonte vietata - solo il manifesto lo e'). (4) Documento_Gladio_Memoriale_di_un_Gladiatore_blog.mht: 'Memoriale di un Gladiatore, missioni segrete estere', da BLOG (fisicamente.blog, 2023). GRADO C CON RISERVA DI ATTENDIBILITA': fonte auto-pubblicata, non verificabile, riconducibile a un blog - reperto di livello C, da trattare con la stessa cautela delle liste anonime della voce 62.</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: ATTO DI RICEZIONE con GRADAZIONE DIFFERENZIATA (non tutte le fonti sono uguali - dall'atto parlamentare A al blog C). fonti/ NON era vuota: gia' conteneva biografie Genovese, nazisti in Sudamerica/USA, network finanziario Sudafrica, un censimento fonti P2 (Governali) - queste 4 vi si aggiungono. L'articolo di stampa e il memoriale-blog restano fonti da usare con cautela (allegazione, non prova); il saggio Cross e l'atto De Luca sono fonti di prim'ordine per il caso Cirillo e la Camorra. Nessuna interrogazione in rete. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>RICEZIONE FONTI CERTIFICATA (4 fonti primarie graduate: parlamentare A/B, accademica B, stampa B/C, blog C). Domini: D7 (stragi/Gladio), D1 (Camorra), D4 (P2).</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>fonti/ (Memoria_Condivisa De Luca; Storiaememoria/caso Cirillo; Due_agosto la Repubblica; Memoriale_Gladiatore blog)</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Triangolazione totale del lotto: 2000 blocchi mirati su nove documenti (voce 75)
Architettura a strati: 90 sintesi mirate (manuali) + 1.228 blocchi di
triangolazione capoverso-per-capoverso contro l'intero grafo del corpus
+ 162 ponti documento-nodo + 299 sinapsi documentali nuove (coppie
co-occorrenti = archi candidati) + 201 unita' interne certificate + 20
di metodo/verdetto. Tesi recepite: biforcazione delle filiere eversive
(criterio di demarcazione per la tesi bicefala); ODESSA costruzione
postuma; inversione ONU Namibia 1976-77 (come domanda); chiasmo
portoghese; Stati Zero della scheda Trump-Gorbaciov.

Copertura: 819 agganci documentali, 904 innesti puri dichiarati
(materia nuova candidata a nodi futuri). 2000 esatti: A 273, B 819,
C 904, neg 4. Registro a voce 75.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J75"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3811,6 +3811,51 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE TOTALE DEL LOTTO (voce 74) con 2000 BLOCCHI MIRATI ESATTI - nove documenti, capoverso per capoverso, contro l'intero grafo del corpus - DOCX + Excel a 25 fogli</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica (DOCX) + repertorio (Excel, 2000 blocchi)</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Architettura a strati: 90 blocchi di SINTESI MIRATA (10 per documento, manuali); 1.228 blocchi di TRIANGOLAZIONE AUTOMATICA (ogni capoverso sostanziale cercato contro 486 schede-nodo + 547 capi del connettoma + alias curati); 162 PONTI documento-nodo (con grado sinaptico); 299 SINAPSI DOCUMENTALI NUOVE (coppie di entita' co-occorrenti nello stesso capoverso = archi candidati per il connettoma); 201 UNITA' INTERNE CERTIFICATE (intestazioni di blocco/capitolo/fase); 20 blocchi di metodo e verdetto. TESI MAGGIORI RECEPITE: biforcazione delle filiere eversive + confutazione del monolite dell'Internazionale Nera (Camera Istruttoria - converge con la tesi bicefala, voce 60, e le da' il criterio di demarcazione); ODESSA come costruzione postuma e il pattern unico Paperclip/Osoaviakhim (Diaspora); INVERSIONE dei voti italiani sulla Namibia 1976-77 (ONU - coincidenza col quadro interno registrata come DOMANDA, grado C); il chiasmo portoghese (protegge Aginter, sorveglia l'Opus Dei); i tre Stati Zero della scheda Trump-Gorbaciov (sosia 1988).</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>ESITO DELLA COPERTURA: 819 blocchi con AGGANCIO documentale al corpus (il lotto parla ai nodi esistenti: Evola/Freda/Rauti, Barbie e i teatri, Aginter/Guerin-Serac, dorsale apartheid, Moro/Santa Sede); 904 INNESTI PURI (capoversi senza aggancio = materia nuova: catena Brighton Beach, personale della diaspora, canali onusiani - candidati a nodi futuri); le 299 coppie co-occorrenti sono la mappa pronta dei nuovi archi. Sezione esoterica + monografia del Sacro federate a vicenda col divieto di inferenza simbolica e i falsificatori designati; Quarta serie = gemello d'autore del registro delle verifiche (linea V61-V70 cumulativa attestata per struttura).</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: triangolazione su SOLO corpus + lotto, nessuna interrogazione in rete; grana lessicale degli strati automatici dichiarata e compensata dagli strati manuali; innesti puri dichiarati C (non forzati); negativi registrati (documento atteso QUINTO_REGISTRO; PDF Sacro atteso; pendenze interne della Quarta serie: Oder-Neisse, ricognizione keniota, cinque proposizioni, linea speculare). Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE TOTALE ESEGUITA (2000 blocchi esatti: A 273, B 819, C 904, neg 4; 25 fogli). Il lotto entra FEDERATO, non giustapposto. Domini: D2, D3, D4, D5, D6, D7, D8 + MONDO NERO.</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica/ITALIA_NERA_TRIANGOLAZIONE_LOTTO_2000_BLOCCHI.docx + repertorio/ITALIA_NERA_TRIANGOLAZIONE_LOTTO_2000_BLOCCHI.xlsx</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atto di ricezione del secondo lotto: 6 nuovi documenti (voce 76)
Nuovi: Tomo V.2 parlamentare "La dimensione sovranazionale del fenomeno
eversivo" (~121k parole, in due varianti -> fonti/); DOSSIER V10 "La
vendetta del Che: Monika Ertl" (50 pp, triangolo Bolivia-Amburgo-Milano);
Rete P2 e dittature (Condor/stronismo/apartheid); Diaspora nazista PDF
(base di ricerca della Sezione); rapporto Ilan Shor (guerra ibrida
2024-26, Mondo Nero contemporaneo). Ri-allegati gia' in corpus
deduplicati (7); doppioni scartati (3). Registro a voce 76.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3856,6 +3856,51 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>ATTO DI RICEZIONE del SECONDO LOTTO: 6 documenti nuovi (2 tomi parlamentari + 4 PDF di ricerca) - 7 ri-allegati gia' in corpus deduplicati, 3 doppioni interni scartati</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>fonti/ (tomi parlamentari) + corpus/opera (PDF di ricerca)</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>NUOVI: (1-2) XIII Legislatura, Doc. XXIII n. 64, Vol. I, TOMO V.2 - 'LA DIMENSIONE SOVRANAZIONALE DEL FENOMENO EVERSIVO IN ITALIA' (Commissione stragi; ~121.000 parole) in DUE VARIANTI con hash diverso (contenuto pressoche' identico: la seconda collocata come _VARIANTE; capitoli: collegamenti internazionali, Apparato di Vigilanza Rivoluzionaria, Orizzontale Latina, Centro Estero, Secchia, rapporto SISMI su Cecoslovacchia/Sejna, carteggio Havel...) -&gt; fonti/, grado A per l'acquisizione (atto parlamentare); (3) ITALIA_NERA_DOSSIER_V10_QUADRANTE_MORO_INTERNAZIONALE.pdf (50 pp, 28.653 parole): 'LA VENDETTA DEL CHE: MONIKA ERTL - il triangolo Bolivia-Amburgo-Milano 1948-1983', quinta campagna del Dossier - 12 capitoli (famiglia Ertl, Quintanilla, ELN/Teoponte, esecuzione di Amburgo 1.4.1971, pista Feltrinelli, apparati attorno a Barbie, summit del crimine Apalachin/Palermo/Montalto, teatro boliviano P2/WACL, Aginter, Hyperion); (4) Rete_P2_E_Dittature_Internazionali_Analisi_Estesa.pdf (18 pp: P2/Condor/stronismo/apartheid, metodologia dell'incrocio onomastico, falsi positivi, Massagrande, Graziani, Paraguay come epicentro); (5) Diaspora_Nazista_PostBellica_Ricerca_Approfondita_1.pdf (40 pp, 10 capitoli: i teatri della diaspora con apparato URL - la base di ricerca della Sezione della voce 74); (6) Ricerca_Oligarca_Ilan_Shor_Connessioni_Internazionali.pdf (21 pp: rapporto sull'infrastruttura di guerra ibrida di Ilan Shor 2024-2026 - MONDO NERO contemporaneo, vettori di infiltrazione, mappatura URL).</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>RI-ALLEGATI GIA' IN CORPUS (deduplicati per hash, nessuna copia doppia): Sezione Diaspora, Italia-ONU Embargo, Nazisti_in_USA_Ricerca_Approfondita.pdf, VERIFICA_03 (Spagna/Portogallo), VERIFICA_05 (Diaspora), VERIFICA_06 (Paperclip), VERIFICA_08 (Sud America) - saranno inclusi nella triangolazione del lotto come richiesto ('tutti i documenti allegati'), i primi due per rinvio alla voce 75 (gia' triangolati capoverso per capoverso). Doppioni interni al lotto scartati: 3. NOTA: il PDF 'Rete P2 e dittature' usa il paradigma dell''Internazionale Nera' che la Camera Istruttoria (voce 74) CONFUTA come monolite: la tensione fra i due documenti d'autore va registrata nella triangolazione, non sanata d'ufficio.</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: ATTO DI RICEZIONE con deduplica per hash e nomi puliti; tomo parlamentare = A per l'acquisizione, B per le valutazioni (undicesima regola della risalita); PDF di ricerca = B (con apparati URL da censire); Shor = MONDO NERO contemporaneo, B/C. Nessuna interrogazione in rete. Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>RICEZIONE CERTIFICATA (6 nuovi + 7 ri-allegati dedup + 3 doppioni scartati). Domini: D7, D2, D3, D4, D9 + MONDO NERO. Prossimo atto: triangolazione del lotto con 2000 blocchi (voce 77).</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>fonti/ (Tomo V.2 + variante) + corpus/opera/ (4 PDF)</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Voce 77: triangolazione totale del secondo lotto con 2000 blocchi mirati esatti (13 documenti, 29 fogli)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3901,6 +3901,51 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE TOTALE DEL SECONDO LOTTO (voce 76) con 2000 BLOCCHI MIRATI ESATTI - tredici documenti, capoverso per capoverso, contro l'intero grafo del corpus - DOCX + Excel a 29 fogli</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica (DOCX) + repertorio (Excel, 2000 blocchi)</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Architettura a strati: 130 blocchi di SINTESI MIRATA (10 per documento, manuali); 1.592 blocchi di TRIANGOLAZIONE AUTOMATICA (ogni capoverso sostanziale vs 486 schede-nodo + connettoma + alias curati); 195 PONTI documento-nodo; 63 SINAPSI DOCUMENTALI NUOVE (coppie co-occorrenti = archi candidati); 20 blocchi di metodo e verdetto. CAMPIONAMENTO DICHIARATO sul Tomo V.2 (XIII leg., Doc. XXIII n.64, Vol. I, ~121.000 parole): 1 capoverso ogni 2 (719 su 1.437) - copertura fine a future unita' dedicate, testo integrale in fonti/; variante non ricontata (collazione = pendenza). TESI MAGGIORI: dimensione sovranazionale parlamentare (Apparato di Vigilanza Rivoluzionaria, Centro Estero/Secchia, rapporto SISMI-Cecoslovacchia/Sejna, carteggio Havel); quadrante andino (Monika Ertl, triangolo Bolivia-Amburgo-Milano: il documento piu' agganciato del lotto, 255/372 capoversi con aggancio); Paraguay epicentro della transumanza nera; TENSIONE REGISTRATA 'Internazionale Nera' (PDF P2-dittature) vs confutazione del monolite (Camera, voce 74) - prevale per statuto il criterio della Camera; Mondo Nero contemporaneo (Shor: 4/99 agganci = innesto quasi puro).</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>ESITO DELLA COPERTURA: 502 blocchi con AGGANCIO documentale (Barbie, Feltrinelli, Aginter, i teatri della diaspora, i vertici criminali) e 1.090 INNESTI PURI - proporzione piu' spostata verso l'innesto rispetto al lotto 1 per il personale nuovo del tomo parlamentare (apparati dell'Est) e per la contemporaneita' del rapporto Shor; il caso boliviano risulta attestato da QUATTRO strati concordi (V10 + Barbie + Verifica 08 + Sezione), il fronte USA e l'iberico da tre. Le 63 coppie co-occorrenti sono la mappa dei nuovi archi.</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: triangolazione su SOLO corpus + lotto, nessuna interrogazione in rete; campionamento dichiarato con k esplicito; grana lessicale degli strati automatici dichiarata e compensata dagli strati manuali; innesti puri non forzati (grado C); negativi registrati (variante non ricontata; pendenze interne delle verifiche). Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE TOTALE ESEGUITA (2000 blocchi esatti: A 65, B 838, C 1.091, neg 6; 29 fogli). Il secondo lotto entra FEDERATO, non giustapposto. Domini: D2, D3, D4, D7 + MONDO NERO + dimensione sovranazionale.</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica/ITALIA_NERA_TRIANGOLAZIONE_LOTTO2_2000_BLOCCHI.docx + repertorio/ITALIA_NERA_TRIANGOLAZIONE_LOTTO2_2000_BLOCCHI.xlsx</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Voci 78-79: ricezione e triangolazione del terzo lotto (Russia Unita/Zheleznyak, 152 blocchi, omonimie scartate)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
+++ b/corpus/diagnostica/ITALIA_NERA_REGISTRO_VERIFICHE_DOCUMENTALI.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J78"/>
+  <dimension ref="A1:J80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3946,6 +3946,96 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>ATTO DI RICEZIONE del TERZO LOTTO: 16 file conferiti - deduplica per impronta E per contenuto: 1 NUOVO, 2 varianti di formato, 1 doppione di contenuto con hash diverso, 12 doppioni per hash scartati</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera (nuovo + varianti)</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>NUOVO: Russia_Unita_Accordi_Internazionali_e_Zheleznyak.pdf (16 pp, ~6.400 parole): 'L'Internazionale Parallela' - la diplomazia partitica di Russia Unita e la guerra cognitiva globale sotto la regia di Sergei Zheleznyak (sanzionato per la Crimea); la rete dei 58 accordi fra partiti col paradigma dell'accordo di Mosca 6.3.2017 con la Lega Nord; Italia 'laboratorio', Austria, Balcani (Dichiarazione di Lovcen), spazio post-sovietico, Sud Globale -&gt; MONDO NERO, secondo pilastro accanto al rapporto Shor (voce 76). VARIANTI DI FORMATO collocate accanto ai primari: Nazisti_in_USA_Ricerca_Approfondita.txt e Nazisti_in_URSS_Ricerca_Approfondita.docx (testo identico ai PDF gia' in corpus, verificato su inizio/fine/capitoli).</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>NAZIINUSA.pdf: impronta NUOVA ma contenuto IDENTICO al finding aid gia' in fonti/ (stesso inizio, stessa fine, stesse 537 parole) -&gt; DOPPIONE DI CONTENUTO scartato: fissata la regola che due impronte diverse possono custodire lo stesso testo (confronto testuale d'obbligo). 12 doppioni per hash scartati (fra cui 2 doppi anche interni al lotto); rilevata pendenza di pulizia: Diaspora_Nazista_..._Approfondita.docx figura in corpus in DUE copie identiche.</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: deduplica dichiarata file per file nel foglio 'Ricezione e deduplica' del repertorio del lotto; nessuna interrogazione in rete; vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>RICEZIONE CERTIFICATA (1 nuovo + 2 varianti + 13 scarti dichiarati). Dominio: MONDO NERO. Prossimo atto: triangolazione del lotto (voce 79).</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>corpus/opera/ (3 file collocati)</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE DEL TERZO LOTTO con 152 BLOCCHI - il rapporto Russia Unita/Zheleznyak capoverso per capoverso, il finding aid campionato, le omonimie scartate - DOCX + Excel a 9 fogli</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica (DOCX) + repertorio (Excel, 152 blocchi)</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Architettura: 16 blocchi di ricezione/deduplica; 10 di sintesi mirata; 98 di TRIANGOLAZIONE AUTOMATICA (capoverso per capoverso vs 486 schede-nodo + connettoma + alias): 2 SOLI AGGANCI GENUINI (Putin; Namibia/SWAPO) e 96 innesti puri - il corpus storico si ferma ai primi anni '90, il rapporto e' materia contemporanea; 3 ponti documento-nodo + 2 FALSI POSITIVI dichiarati; 1 sinapsi documentale nuova (Namibia&lt;-&gt;SWAPO); 10 blocchi di campione del finding aid (Cukurs, Arajs, Artukovic, Axmann, d'Alquen - con difetto di lezione da traduzione automatica dichiarato); 10 di statuto e verdetto. CONVERGENZA REGISTRATA: la SWAPO della rete di Russia Unita e' la stessa Namibia dell'inversione dei voti italiani 1976-77 (voce 75) - continuita' di TEATRO come dato, nessuna inferenza di continuita' di regia.</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>ESITO PIU' ISTRUTTIVO: l'aggancio automatico proponeva 'Partito Democratico' e 'Partito Repubblicano' (nodi del corpus), ma la lettura dei contesti mostra che designano il Partito Democratico di Serbia, il PDP-Laban filippino, il Partito Repubblicano d'Armenia, il PDP tagiko: OMONIMIE = falsi positivi dell'incrocio onomastico, scartati e registrati - PRIMA APPLICAZIONE OPERATIVA della metodologia dei falsi positivi teorizzata dal PDF Rete_P2_E_Dittature (voce 76): il lotto precedente ha fornito la regola con cui si e' vagliato il successivo.</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Statuto: triangolazione su SOLO corpus + lotto; omonimie scartate per lettura dei contesti; l'elenco nominativo indirizza e non pronuncia; negativi registrati (lezione deformata del finding aid; doppia copia interna Diaspora; materia contemporanea che aggancia poco per costruzione). Vincolo fonti rispettato (no Grokipedia, no il manifesto).</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>TRIANGOLAZIONE ESEGUITA (152 blocchi: A 16, B 24, C 96, neg 16; 9 fogli). Il terzo lotto entra FEDERATO. Catena ricezione-triangolazione = protocollo stabile (74-75, 76-77, 78-79). Dominio: MONDO NERO + D.diaspora.</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>corpus/diagnostica/ITALIA_NERA_TRIANGOLAZIONE_LOTTO3_RUSSIA_UNITA.docx + repertorio/ITALIA_NERA_TRIANGOLAZIONE_LOTTO3_RUSSIA_UNITA.xlsx</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>9.8.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>